<commit_message>
data: populate guanghe REIT monthly operational data (37 months, 2023-06~2026-06)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -1124,7 +1124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1180,166 +1180,1260 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6854</v>
+      </c>
+      <c r="E2" t="n">
+        <v>151484</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8133</v>
+      </c>
+      <c r="E3" t="n">
+        <v>162665</v>
+      </c>
+      <c r="F3" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>8391</v>
+      </c>
+      <c r="E4" t="n">
+        <v>164090</v>
+      </c>
+      <c r="F4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6626</v>
+      </c>
+      <c r="E5" t="n">
+        <v>138230</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5590</v>
+      </c>
+      <c r="E6" t="n">
+        <v>118420</v>
+      </c>
+      <c r="F6" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6720</v>
+      </c>
+      <c r="E7" t="n">
+        <v>147610</v>
+      </c>
+      <c r="F7" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7068</v>
+      </c>
+      <c r="E8" t="n">
+        <v>150397</v>
+      </c>
+      <c r="F8" t="n">
+        <v>42</v>
+      </c>
+      <c r="G8" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7389</v>
+      </c>
+      <c r="E9" t="n">
+        <v>151350</v>
+      </c>
+      <c r="F9" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>5324</v>
+      </c>
+      <c r="E10" t="n">
+        <v>112154</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-21.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-27.2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6529</v>
+      </c>
+      <c r="E11" t="n">
+        <v>143579</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-3.2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5715</v>
+      </c>
+      <c r="E12" t="n">
+        <v>127791</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-11.6</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5318</v>
+      </c>
+      <c r="E13" t="n">
+        <v>115499</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-8.9</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-10.1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6222</v>
+      </c>
+      <c r="E14" t="n">
+        <v>142379</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-9.199999999999999</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-6</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>7198</v>
+      </c>
+      <c r="E15" t="n">
+        <v>150597</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-11.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-7.4</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>7615</v>
+      </c>
+      <c r="E16" t="n">
+        <v>155032</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-9.25</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-5.52</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6724</v>
+      </c>
+      <c r="E17" t="n">
+        <v>149596</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="G17" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>5343</v>
+      </c>
+      <c r="E18" t="n">
+        <v>112156</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-4.41</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-5.29</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>6363</v>
+      </c>
+      <c r="E19" t="n">
+        <v>143976</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-5.31</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>6792</v>
+      </c>
+      <c r="E20" t="n">
+        <v>145349</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-3.91</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-3.36</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>2025-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>180201</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>平安广州广河REIT</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>8256</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>128500</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>月度运营公告</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>7104</v>
+      </c>
+      <c r="E21" t="n">
+        <v>135187</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-3.86</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-10.68</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>2025-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>180201</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>平安广州广河REIT</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>7200</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>115000</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>-2.1</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>月度运营公告</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5188</v>
+      </c>
+      <c r="E22" t="n">
+        <v>126701</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-2.55</v>
+      </c>
+      <c r="G22" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>2025-03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>180201</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>平安广州广河REIT</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>8900</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>135000</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>月度运营公告</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6530</v>
+      </c>
+      <c r="E23" t="n">
+        <v>141180</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-1.67</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>2025-04</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>180201</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>平安广州广河REIT</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>8300</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>130000</v>
-      </c>
-      <c r="F5" s="6" t="n">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5702</v>
+      </c>
+      <c r="E24" t="n">
+        <v>129326</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="G24" t="n">
         <v>1.2</v>
       </c>
-      <c r="G5" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>月度运营公告</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>📝 填写说明：</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>• 每只REIT每月一条数据，来自交易所"月度主要运营数据公告"</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>• 通行费收入和日均车流量为核心指标，同比数据如公告中有则填写</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>• 报告期格式：YYYY-MM（如2025-01）</t>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>5558</v>
+      </c>
+      <c r="E25" t="n">
+        <v>122526</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6336</v>
+      </c>
+      <c r="E26" t="n">
+        <v>146421</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>7203</v>
+      </c>
+      <c r="E27" t="n">
+        <v>153916</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>7342</v>
+      </c>
+      <c r="E28" t="n">
+        <v>152327</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>6020</v>
+      </c>
+      <c r="E29" t="n">
+        <v>137485</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-10.47</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>5232</v>
+      </c>
+      <c r="E30" t="n">
+        <v>109238</v>
+      </c>
+      <c r="F30" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>6166</v>
+      </c>
+      <c r="E31" t="n">
+        <v>139016</v>
+      </c>
+      <c r="F31" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-3.45</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>6693</v>
+      </c>
+      <c r="E32" t="n">
+        <v>143816</v>
+      </c>
+      <c r="F32" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-1.05</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>7002</v>
+      </c>
+      <c r="E33" t="n">
+        <v>153265</v>
+      </c>
+      <c r="F33" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="G33" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>5397</v>
+      </c>
+      <c r="E34" t="n">
+        <v>118608</v>
+      </c>
+      <c r="F34" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-6.39</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>6640</v>
+      </c>
+      <c r="E35" t="n">
+        <v>148905</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="G35" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>5571</v>
+      </c>
+      <c r="E36" t="n">
+        <v>133697</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="G36" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5258</v>
+      </c>
+      <c r="E37" t="n">
+        <v>121008</v>
+      </c>
+      <c r="F37" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="G37" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>6106</v>
+      </c>
+      <c r="E38" t="n">
+        <v>147050</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-3.63</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: populate SZ REITs monthly data (180201/180202/180203, 94 rows)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -1124,7 +1124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1180,7 +1180,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
@@ -1214,67 +1214,67 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E3" t="n">
+        <v>32745</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>7</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>180201</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>平安广州广河REIT</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>8133</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E4" t="n">
         <v>162665</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F4" t="n">
         <v>13.3</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G4" t="n">
         <v>12.3</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>月度运营公告（自动采集）</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>2023-08</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>180201</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>平安广州广河REIT</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>8391</v>
-      </c>
-      <c r="E4" t="n">
-        <v>164090</v>
-      </c>
-      <c r="F4" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="G4" t="n">
-        <v>9.4</v>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>月度运营公告（自动采集）</t>
@@ -1282,32 +1282,32 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>2023-09</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2023-07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6626</v>
+        <v>2172</v>
       </c>
       <c r="E5" t="n">
-        <v>138230</v>
+        <v>34542</v>
       </c>
       <c r="F5" t="n">
-        <v>1.7</v>
+        <v>14.3</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.9</v>
+        <v>10.7</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1332,16 +1332,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5590</v>
+        <v>8391</v>
       </c>
       <c r="E6" t="n">
-        <v>118420</v>
+        <v>164090</v>
       </c>
       <c r="F6" t="n">
-        <v>19.4</v>
+        <v>12.5</v>
       </c>
       <c r="G6" t="n">
-        <v>24.2</v>
+        <v>9.4</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1352,30 +1352,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6720</v>
+        <v>2289</v>
       </c>
       <c r="E7" t="n">
-        <v>147610</v>
+        <v>37112</v>
       </c>
       <c r="F7" t="n">
-        <v>63.5</v>
+        <v>21.4</v>
       </c>
       <c r="G7" t="n">
-        <v>65.90000000000001</v>
+        <v>22</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1400,16 +1400,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7068</v>
+        <v>6626</v>
       </c>
       <c r="E8" t="n">
-        <v>150397</v>
+        <v>138230</v>
       </c>
       <c r="F8" t="n">
-        <v>42</v>
+        <v>1.7</v>
       </c>
       <c r="G8" t="n">
-        <v>45.8</v>
+        <v>-1.9</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1420,30 +1420,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7389</v>
+        <v>2014</v>
       </c>
       <c r="E9" t="n">
-        <v>151350</v>
+        <v>31714</v>
       </c>
       <c r="F9" t="n">
-        <v>13.3</v>
+        <v>19.7</v>
       </c>
       <c r="G9" t="n">
-        <v>24.9</v>
+        <v>24</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1454,7 +1454,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1468,16 +1468,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5324</v>
+        <v>5590</v>
       </c>
       <c r="E10" t="n">
-        <v>112154</v>
+        <v>118420</v>
       </c>
       <c r="F10" t="n">
-        <v>-21.1</v>
+        <v>19.4</v>
       </c>
       <c r="G10" t="n">
-        <v>-27.2</v>
+        <v>24.2</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1488,30 +1488,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6529</v>
+        <v>1701</v>
       </c>
       <c r="E11" t="n">
-        <v>143579</v>
+        <v>25397</v>
       </c>
       <c r="F11" t="n">
-        <v>-3.2</v>
+        <v>32</v>
       </c>
       <c r="G11" t="n">
-        <v>-1</v>
+        <v>49</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1522,7 +1522,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1536,16 +1536,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5715</v>
+        <v>6720</v>
       </c>
       <c r="E12" t="n">
-        <v>127791</v>
+        <v>147610</v>
       </c>
       <c r="F12" t="n">
-        <v>-11.6</v>
+        <v>63.5</v>
       </c>
       <c r="G12" t="n">
-        <v>-4.6</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1556,30 +1556,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5318</v>
+        <v>1970</v>
       </c>
       <c r="E13" t="n">
-        <v>115499</v>
+        <v>31356</v>
       </c>
       <c r="F13" t="n">
-        <v>-8.9</v>
+        <v>47.7</v>
       </c>
       <c r="G13" t="n">
-        <v>-10.1</v>
+        <v>82.8</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1590,7 +1590,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1604,16 +1604,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6222</v>
+        <v>7068</v>
       </c>
       <c r="E14" t="n">
-        <v>142379</v>
+        <v>150397</v>
       </c>
       <c r="F14" t="n">
-        <v>-9.199999999999999</v>
+        <v>42</v>
       </c>
       <c r="G14" t="n">
-        <v>-6</v>
+        <v>45.8</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1624,30 +1624,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7198</v>
+        <v>2001</v>
       </c>
       <c r="E15" t="n">
-        <v>150597</v>
+        <v>31076</v>
       </c>
       <c r="F15" t="n">
-        <v>-11.5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G15" t="n">
-        <v>-7.4</v>
+        <v>-1.3</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1658,7 +1658,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1672,16 +1672,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7615</v>
+        <v>7389</v>
       </c>
       <c r="E16" t="n">
-        <v>155032</v>
+        <v>151350</v>
       </c>
       <c r="F16" t="n">
-        <v>-9.25</v>
+        <v>13.3</v>
       </c>
       <c r="G16" t="n">
-        <v>-5.52</v>
+        <v>24.9</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1692,30 +1692,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6724</v>
+        <v>2188</v>
       </c>
       <c r="E17" t="n">
-        <v>149596</v>
+        <v>36106</v>
       </c>
       <c r="F17" t="n">
-        <v>1.47</v>
+        <v>-2</v>
       </c>
       <c r="G17" t="n">
-        <v>8.220000000000001</v>
+        <v>-9.1</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1726,7 +1726,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1740,16 +1740,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5343</v>
+        <v>5324</v>
       </c>
       <c r="E18" t="n">
-        <v>112156</v>
+        <v>112154</v>
       </c>
       <c r="F18" t="n">
-        <v>-4.41</v>
+        <v>-21.1</v>
       </c>
       <c r="G18" t="n">
-        <v>-5.29</v>
+        <v>-27.2</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1760,30 +1760,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6363</v>
+        <v>1463</v>
       </c>
       <c r="E19" t="n">
-        <v>143976</v>
+        <v>29163</v>
       </c>
       <c r="F19" t="n">
-        <v>-5.31</v>
+        <v>-32.2</v>
       </c>
       <c r="G19" t="n">
-        <v>-2.46</v>
+        <v>-26.5</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1794,7 +1794,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1808,16 +1808,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6792</v>
+        <v>6529</v>
       </c>
       <c r="E20" t="n">
-        <v>145349</v>
+        <v>143579</v>
       </c>
       <c r="F20" t="n">
-        <v>-3.91</v>
+        <v>-3.2</v>
       </c>
       <c r="G20" t="n">
-        <v>-3.36</v>
+        <v>-1</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1828,30 +1828,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>7104</v>
+        <v>2132</v>
       </c>
       <c r="E21" t="n">
-        <v>135187</v>
+        <v>34630</v>
       </c>
       <c r="F21" t="n">
-        <v>-3.86</v>
+        <v>2.6</v>
       </c>
       <c r="G21" t="n">
-        <v>-10.68</v>
+        <v>11.1</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1862,7 +1862,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1876,16 +1876,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5188</v>
+        <v>5715</v>
       </c>
       <c r="E22" t="n">
-        <v>126701</v>
+        <v>127791</v>
       </c>
       <c r="F22" t="n">
-        <v>-2.55</v>
+        <v>-11.6</v>
       </c>
       <c r="G22" t="n">
-        <v>12.97</v>
+        <v>-4.6</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1896,30 +1896,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6530</v>
+        <v>1916</v>
       </c>
       <c r="E23" t="n">
-        <v>141180</v>
+        <v>31433</v>
       </c>
       <c r="F23" t="n">
-        <v>0.02</v>
+        <v>0.4</v>
       </c>
       <c r="G23" t="n">
-        <v>-1.67</v>
+        <v>4.7</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1944,16 +1944,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5702</v>
+        <v>5318</v>
       </c>
       <c r="E24" t="n">
-        <v>129326</v>
+        <v>115499</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.22</v>
+        <v>-8.9</v>
       </c>
       <c r="G24" t="n">
-        <v>1.2</v>
+        <v>-10.1</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1964,30 +1964,30 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5558</v>
+        <v>1741</v>
       </c>
       <c r="E25" t="n">
-        <v>122526</v>
+        <v>27355</v>
       </c>
       <c r="F25" t="n">
-        <v>4.51</v>
+        <v>-4.1</v>
       </c>
       <c r="G25" t="n">
-        <v>6.08</v>
+        <v>2.4</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2012,16 +2012,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6336</v>
+        <v>6222</v>
       </c>
       <c r="E26" t="n">
-        <v>146421</v>
+        <v>142379</v>
       </c>
       <c r="F26" t="n">
-        <v>1.84</v>
+        <v>-9.199999999999999</v>
       </c>
       <c r="G26" t="n">
-        <v>2.84</v>
+        <v>-6</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2032,30 +2032,30 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7203</v>
+        <v>1952</v>
       </c>
       <c r="E27" t="n">
-        <v>153916</v>
+        <v>34158</v>
       </c>
       <c r="F27" t="n">
-        <v>0.06</v>
+        <v>-3.2</v>
       </c>
       <c r="G27" t="n">
-        <v>2.2</v>
+        <v>4.3</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -2066,7 +2066,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2080,16 +2080,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>7342</v>
+        <v>7198</v>
       </c>
       <c r="E28" t="n">
-        <v>152327</v>
+        <v>150597</v>
       </c>
       <c r="F28" t="n">
-        <v>-3.58</v>
+        <v>-11.5</v>
       </c>
       <c r="G28" t="n">
-        <v>-1.75</v>
+        <v>-7.4</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -2100,30 +2100,30 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>6020</v>
+        <v>1987</v>
       </c>
       <c r="E29" t="n">
-        <v>137485</v>
+        <v>34418</v>
       </c>
       <c r="F29" t="n">
-        <v>-10.47</v>
+        <v>-8.5</v>
       </c>
       <c r="G29" t="n">
-        <v>-8.1</v>
+        <v>-0.4</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -2134,7 +2134,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2148,16 +2148,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5232</v>
+        <v>7615</v>
       </c>
       <c r="E30" t="n">
-        <v>109238</v>
+        <v>155032</v>
       </c>
       <c r="F30" t="n">
-        <v>-2.09</v>
+        <v>-9.25</v>
       </c>
       <c r="G30" t="n">
-        <v>-2.6</v>
+        <v>-5.52</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -2168,30 +2168,30 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6166</v>
+        <v>2128</v>
       </c>
       <c r="E31" t="n">
-        <v>139016</v>
+        <v>37205</v>
       </c>
       <c r="F31" t="n">
-        <v>-3.1</v>
+        <v>-7.1</v>
       </c>
       <c r="G31" t="n">
-        <v>-3.45</v>
+        <v>0.2</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -2202,7 +2202,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2216,16 +2216,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>6693</v>
+        <v>6724</v>
       </c>
       <c r="E32" t="n">
-        <v>143816</v>
+        <v>149596</v>
       </c>
       <c r="F32" t="n">
-        <v>-1.46</v>
+        <v>1.47</v>
       </c>
       <c r="G32" t="n">
-        <v>-1.05</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -2236,30 +2236,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7002</v>
+        <v>1914</v>
       </c>
       <c r="E33" t="n">
-        <v>153265</v>
+        <v>34369</v>
       </c>
       <c r="F33" t="n">
-        <v>-1.44</v>
+        <v>-5</v>
       </c>
       <c r="G33" t="n">
-        <v>13.37</v>
+        <v>8.4</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2270,7 +2270,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2284,16 +2284,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5397</v>
+        <v>5343</v>
       </c>
       <c r="E34" t="n">
-        <v>118608</v>
+        <v>112156</v>
       </c>
       <c r="F34" t="n">
-        <v>4.04</v>
+        <v>-4.41</v>
       </c>
       <c r="G34" t="n">
-        <v>-6.39</v>
+        <v>-5.29</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2304,30 +2304,30 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6640</v>
+        <v>1561</v>
       </c>
       <c r="E35" t="n">
-        <v>148905</v>
+        <v>25194</v>
       </c>
       <c r="F35" t="n">
-        <v>1.68</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="G35" t="n">
-        <v>5.47</v>
+        <v>-0.8</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2338,7 +2338,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2352,16 +2352,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>5571</v>
+        <v>6363</v>
       </c>
       <c r="E36" t="n">
-        <v>133697</v>
+        <v>143976</v>
       </c>
       <c r="F36" t="n">
-        <v>-2.29</v>
+        <v>-5.31</v>
       </c>
       <c r="G36" t="n">
-        <v>3.38</v>
+        <v>-2.46</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2372,30 +2372,30 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>180201</t>
+          <t>180202</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>平安广州广河REIT</t>
+          <t>华夏越秀高速REIT</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>5258</v>
+        <v>1834</v>
       </c>
       <c r="E37" t="n">
-        <v>121008</v>
+        <v>31830</v>
       </c>
       <c r="F37" t="n">
-        <v>-5.4</v>
+        <v>-6.9</v>
       </c>
       <c r="G37" t="n">
-        <v>-1.24</v>
+        <v>1.5</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2406,32 +2406,1970 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>14334</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3470</v>
+      </c>
+      <c r="G38" t="n">
+        <v>13462</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>6792</v>
+      </c>
+      <c r="E39" t="n">
+        <v>145349</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-3.91</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-3.36</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1936</v>
+      </c>
+      <c r="E40" t="n">
+        <v>32762</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="G40" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>14071</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F41" t="n">
+        <v>3777</v>
+      </c>
+      <c r="G41" t="n">
+        <v>13335</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>7104</v>
+      </c>
+      <c r="E42" t="n">
+        <v>135187</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-3.86</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-10.68</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>2340</v>
+      </c>
+      <c r="E43" t="n">
+        <v>43779</v>
+      </c>
+      <c r="F43" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G43" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>20086</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4357</v>
+      </c>
+      <c r="G44" t="n">
+        <v>20086</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>5188</v>
+      </c>
+      <c r="E45" t="n">
+        <v>126701</v>
+      </c>
+      <c r="F45" t="n">
+        <v>-2.55</v>
+      </c>
+      <c r="G45" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1780</v>
+      </c>
+      <c r="E46" t="n">
+        <v>37043</v>
+      </c>
+      <c r="F46" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="G46" t="n">
+        <v>27</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>18278</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F47" t="n">
+        <v>3009</v>
+      </c>
+      <c r="G47" t="n">
+        <v>16277</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>6530</v>
+      </c>
+      <c r="E48" t="n">
+        <v>141180</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-1.67</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1915</v>
+      </c>
+      <c r="E49" t="n">
+        <v>33112</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-10.2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>16983</v>
+      </c>
+      <c r="E50" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F50" t="n">
+        <v>3776</v>
+      </c>
+      <c r="G50" t="n">
+        <v>14517</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>5702</v>
+      </c>
+      <c r="E51" t="n">
+        <v>129326</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="G51" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1753</v>
+      </c>
+      <c r="E52" t="n">
+        <v>31029</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-8.5</v>
+      </c>
+      <c r="G52" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>16161</v>
+      </c>
+      <c r="E53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F53" t="n">
+        <v>3589</v>
+      </c>
+      <c r="G53" t="n">
+        <v>13697</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>5558</v>
+      </c>
+      <c r="E54" t="n">
+        <v>122526</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="G54" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>1668</v>
+      </c>
+      <c r="E55" t="n">
+        <v>28348</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="G55" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>15559</v>
+      </c>
+      <c r="E56" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F56" t="n">
+        <v>3569</v>
+      </c>
+      <c r="G56" t="n">
+        <v>13116</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>6336</v>
+      </c>
+      <c r="E57" t="n">
+        <v>146421</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="G57" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1802</v>
+      </c>
+      <c r="E58" t="n">
+        <v>32947</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>15326</v>
+      </c>
+      <c r="E59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F59" t="n">
+        <v>3508</v>
+      </c>
+      <c r="G59" t="n">
+        <v>14153</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>7203</v>
+      </c>
+      <c r="E60" t="n">
+        <v>153916</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G60" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>1962</v>
+      </c>
+      <c r="E61" t="n">
+        <v>35097</v>
+      </c>
+      <c r="F61" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="G61" t="n">
+        <v>2</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>15371</v>
+      </c>
+      <c r="E62" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F62" t="n">
+        <v>3867</v>
+      </c>
+      <c r="G62" t="n">
+        <v>15634</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>7342</v>
+      </c>
+      <c r="E63" t="n">
+        <v>152327</v>
+      </c>
+      <c r="F63" t="n">
+        <v>-3.58</v>
+      </c>
+      <c r="G63" t="n">
+        <v>-1.75</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>2127</v>
+      </c>
+      <c r="E64" t="n">
+        <v>38625</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>15601</v>
+      </c>
+      <c r="E65" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F65" t="n">
+        <v>4087</v>
+      </c>
+      <c r="G65" t="n">
+        <v>17173</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>6020</v>
+      </c>
+      <c r="E66" t="n">
+        <v>137485</v>
+      </c>
+      <c r="F66" t="n">
+        <v>-10.47</v>
+      </c>
+      <c r="G66" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>1827</v>
+      </c>
+      <c r="E67" t="n">
+        <v>33012</v>
+      </c>
+      <c r="F67" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="G67" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>15637</v>
+      </c>
+      <c r="E68" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F68" t="n">
+        <v>3962</v>
+      </c>
+      <c r="G68" t="n">
+        <v>15930</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>5232</v>
+      </c>
+      <c r="E69" t="n">
+        <v>109238</v>
+      </c>
+      <c r="F69" t="n">
+        <v>-2.09</v>
+      </c>
+      <c r="G69" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1520</v>
+      </c>
+      <c r="E70" t="n">
+        <v>25101</v>
+      </c>
+      <c r="F70" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="G70" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>15371</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F71" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G71" t="n">
+        <v>13033</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>6166</v>
+      </c>
+      <c r="E72" t="n">
+        <v>139016</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="G72" t="n">
+        <v>-3.45</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1831</v>
+      </c>
+      <c r="E73" t="n">
+        <v>32654</v>
+      </c>
+      <c r="F73" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="G73" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>15359</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F74" t="n">
+        <v>4081</v>
+      </c>
+      <c r="G74" t="n">
+        <v>15237</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>6693</v>
+      </c>
+      <c r="E75" t="n">
+        <v>143816</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="G75" t="n">
+        <v>-1.05</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1908</v>
+      </c>
+      <c r="E76" t="n">
+        <v>33245</v>
+      </c>
+      <c r="F76" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>15299</v>
+      </c>
+      <c r="E77" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F77" t="n">
+        <v>3952</v>
+      </c>
+      <c r="G77" t="n">
+        <v>14645</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>7002</v>
+      </c>
+      <c r="E78" t="n">
+        <v>153265</v>
+      </c>
+      <c r="F78" t="n">
+        <v>-1.44</v>
+      </c>
+      <c r="G78" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E79" t="n">
+        <v>35020</v>
+      </c>
+      <c r="F79" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="G79" t="n">
+        <v>-20</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>15880</v>
+      </c>
+      <c r="E80" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F80" t="n">
+        <v>4170</v>
+      </c>
+      <c r="G80" t="n">
+        <v>15880</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>5397</v>
+      </c>
+      <c r="E81" t="n">
+        <v>118608</v>
+      </c>
+      <c r="F81" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="G81" t="n">
+        <v>-6.39</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>1908</v>
+      </c>
+      <c r="E82" t="n">
+        <v>40166</v>
+      </c>
+      <c r="F82" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G82" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>19705</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F83" t="n">
+        <v>4036</v>
+      </c>
+      <c r="G83" t="n">
+        <v>23939</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>6640</v>
+      </c>
+      <c r="E84" t="n">
+        <v>148905</v>
+      </c>
+      <c r="F84" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="G84" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>2179</v>
+      </c>
+      <c r="E85" t="n">
+        <v>39175</v>
+      </c>
+      <c r="F85" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="G85" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>20151</v>
+      </c>
+      <c r="E86" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F86" t="n">
+        <v>4759</v>
+      </c>
+      <c r="G86" t="n">
+        <v>21001</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>5571</v>
+      </c>
+      <c r="E87" t="n">
+        <v>133697</v>
+      </c>
+      <c r="F87" t="n">
+        <v>-2.29</v>
+      </c>
+      <c r="G87" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>1763</v>
+      </c>
+      <c r="E88" t="n">
+        <v>30460</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G88" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>19143</v>
+      </c>
+      <c r="E89" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F89" t="n">
+        <v>4085</v>
+      </c>
+      <c r="G89" t="n">
+        <v>16117</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>180201</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>平安广州广河REIT</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>5258</v>
+      </c>
+      <c r="E90" t="n">
+        <v>121008</v>
+      </c>
+      <c r="F90" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="G90" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>1651</v>
+      </c>
+      <c r="E91" t="n">
+        <v>27250</v>
+      </c>
+      <c r="F91" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="G91" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>18269</v>
+      </c>
+      <c r="E92" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F92" t="n">
+        <v>3949</v>
+      </c>
+      <c r="G92" t="n">
+        <v>14886</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
           <t>2026-06</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>180201</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>平安广州广河REIT</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D93" t="n">
         <v>6106</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E93" t="n">
         <v>147050</v>
       </c>
-      <c r="F38" t="n">
+      <c r="F93" t="n">
         <v>-3.63</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G93" t="n">
         <v>0.43</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>180202</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>华夏越秀高速REIT</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>1916</v>
+      </c>
+      <c r="E94" t="n">
+        <v>34452</v>
+      </c>
+      <c r="F94" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G94" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>月度运营公告（自动采集）</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>180203</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>招商高速公路REIT</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>18073</v>
+      </c>
+      <c r="E95" t="n">
+        <v>2026</v>
+      </c>
+      <c r="F95" t="n">
+        <v>4088</v>
+      </c>
+      <c r="G95" t="n">
+        <v>17086</v>
+      </c>
+      <c r="H95" t="inlineStr">
         <is>
           <t>月度运营公告（自动采集）</t>
         </is>

</xml_diff>

<commit_message>
fix: LABEL_CHARS add 化 (180203 early announcements use 比变化)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -6092,16 +6092,16 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>14334</v>
+        <v>-12.9</v>
       </c>
       <c r="E146" t="n">
-        <v>2024</v>
+        <v>4</v>
       </c>
       <c r="F146" t="n">
-        <v>3470</v>
+        <v>-7.3</v>
       </c>
       <c r="G146" t="n">
-        <v>13462</v>
+        <v>-8.5</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -6466,16 +6466,16 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>14071</v>
+        <v>-4.6</v>
       </c>
       <c r="E157" t="n">
-        <v>2024</v>
+        <v>12</v>
       </c>
       <c r="F157" t="n">
-        <v>3777</v>
+        <v>3.7</v>
       </c>
       <c r="G157" t="n">
-        <v>13335</v>
+        <v>-3.1</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
@@ -6874,16 +6874,16 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>20086</v>
+        <v>36.6</v>
       </c>
       <c r="E169" t="n">
-        <v>2025</v>
+        <v>1</v>
       </c>
       <c r="F169" t="n">
-        <v>4357</v>
+        <v>15.4</v>
       </c>
       <c r="G169" t="n">
-        <v>20086</v>
+        <v>50.6</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
@@ -7282,16 +7282,16 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>18278</v>
+        <v>25.4</v>
       </c>
       <c r="E181" t="n">
-        <v>2025</v>
+        <v>2</v>
       </c>
       <c r="F181" t="n">
-        <v>3009</v>
+        <v>-30.9</v>
       </c>
       <c r="G181" t="n">
-        <v>16277</v>
+        <v>-19</v>
       </c>
       <c r="H181" t="inlineStr">
         <is>
@@ -7724,16 +7724,16 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>16983</v>
+        <v>16.2</v>
       </c>
       <c r="E194" t="n">
-        <v>2025</v>
+        <v>3</v>
       </c>
       <c r="F194" t="n">
-        <v>3776</v>
+        <v>25.5</v>
       </c>
       <c r="G194" t="n">
-        <v>14517</v>
+        <v>-10.8</v>
       </c>
       <c r="H194" t="inlineStr">
         <is>
@@ -8166,16 +8166,16 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>16161</v>
+        <v>12.8</v>
       </c>
       <c r="E207" t="n">
-        <v>2025</v>
+        <v>4</v>
       </c>
       <c r="F207" t="n">
-        <v>3589</v>
+        <v>-5</v>
       </c>
       <c r="G207" t="n">
-        <v>13697</v>
+        <v>-5.6</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
@@ -8608,16 +8608,16 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>15559</v>
+        <v>11.5</v>
       </c>
       <c r="E220" t="n">
-        <v>2025</v>
+        <v>5</v>
       </c>
       <c r="F220" t="n">
-        <v>3569</v>
+        <v>-0.6</v>
       </c>
       <c r="G220" t="n">
-        <v>13116</v>
+        <v>-5</v>
       </c>
       <c r="H220" t="inlineStr">
         <is>
@@ -9050,16 +9050,16 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>15326</v>
+        <v>10.1</v>
       </c>
       <c r="E233" t="n">
-        <v>2025</v>
+        <v>6</v>
       </c>
       <c r="F233" t="n">
-        <v>3508</v>
+        <v>-1.7</v>
       </c>
       <c r="G233" t="n">
-        <v>14153</v>
+        <v>7.9</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
@@ -9492,16 +9492,16 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>15371</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E246" t="n">
-        <v>2025</v>
+        <v>7</v>
       </c>
       <c r="F246" t="n">
-        <v>3867</v>
+        <v>10.2</v>
       </c>
       <c r="G246" t="n">
-        <v>15634</v>
+        <v>10.5</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
@@ -9934,16 +9934,16 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>15601</v>
+        <v>9.4</v>
       </c>
       <c r="E259" t="n">
-        <v>2025</v>
+        <v>8</v>
       </c>
       <c r="F259" t="n">
-        <v>4087</v>
+        <v>5.7</v>
       </c>
       <c r="G259" t="n">
-        <v>17173</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
@@ -10376,16 +10376,16 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>15637</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E272" t="n">
-        <v>2025</v>
+        <v>9</v>
       </c>
       <c r="F272" t="n">
-        <v>3962</v>
+        <v>-3</v>
       </c>
       <c r="G272" t="n">
-        <v>15930</v>
+        <v>-7.2</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
@@ -10818,16 +10818,16 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>15371</v>
+        <v>8.4</v>
       </c>
       <c r="E285" t="n">
-        <v>2025</v>
+        <v>10</v>
       </c>
       <c r="F285" t="n">
-        <v>3680</v>
+        <v>-7.1</v>
       </c>
       <c r="G285" t="n">
-        <v>13033</v>
+        <v>-18.2</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
@@ -11226,16 +11226,16 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>15359</v>
+        <v>8.6</v>
       </c>
       <c r="E297" t="n">
-        <v>2025</v>
+        <v>11</v>
       </c>
       <c r="F297" t="n">
-        <v>4081</v>
+        <v>10.9</v>
       </c>
       <c r="G297" t="n">
-        <v>15237</v>
+        <v>16.9</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
@@ -11634,16 +11634,16 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>15299</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E309" t="n">
-        <v>2025</v>
+        <v>12</v>
       </c>
       <c r="F309" t="n">
-        <v>3952</v>
+        <v>-3.2</v>
       </c>
       <c r="G309" t="n">
-        <v>14645</v>
+        <v>-3.9</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
@@ -12076,16 +12076,16 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>15880</v>
+        <v>-20.9</v>
       </c>
       <c r="E322" t="n">
-        <v>2026</v>
+        <v>1</v>
       </c>
       <c r="F322" t="n">
-        <v>4170</v>
+        <v>5.5</v>
       </c>
       <c r="G322" t="n">
-        <v>15880</v>
+        <v>8.4</v>
       </c>
       <c r="H322" t="inlineStr">
         <is>
@@ -12518,16 +12518,16 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>19705</v>
+        <v>4036</v>
       </c>
       <c r="E335" t="n">
-        <v>2026</v>
+        <v>23939</v>
       </c>
       <c r="F335" t="n">
-        <v>4036</v>
+        <v>34.1</v>
       </c>
       <c r="G335" t="n">
-        <v>23939</v>
+        <v>47.1</v>
       </c>
       <c r="H335" t="inlineStr">
         <is>
@@ -12960,16 +12960,16 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>20151</v>
+        <v>4759</v>
       </c>
       <c r="E348" t="n">
-        <v>2026</v>
+        <v>21001</v>
       </c>
       <c r="F348" t="n">
-        <v>4759</v>
+        <v>26</v>
       </c>
       <c r="G348" t="n">
-        <v>21001</v>
+        <v>44.7</v>
       </c>
       <c r="H348" t="inlineStr">
         <is>
@@ -13402,16 +13402,16 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>19143</v>
+        <v>4085</v>
       </c>
       <c r="E361" t="n">
-        <v>2026</v>
+        <v>16117</v>
       </c>
       <c r="F361" t="n">
-        <v>4085</v>
+        <v>13.8</v>
       </c>
       <c r="G361" t="n">
-        <v>16117</v>
+        <v>16.7</v>
       </c>
       <c r="H361" t="inlineStr">
         <is>
@@ -13878,16 +13878,16 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>18269</v>
+        <v>3949</v>
       </c>
       <c r="E375" t="n">
-        <v>2026</v>
+        <v>14886</v>
       </c>
       <c r="F375" t="n">
-        <v>3949</v>
+        <v>10.6</v>
       </c>
       <c r="G375" t="n">
-        <v>14886</v>
+        <v>13.5</v>
       </c>
       <c r="H375" t="inlineStr">
         <is>
@@ -14354,16 +14354,16 @@
         </is>
       </c>
       <c r="D389" t="n">
-        <v>18073</v>
+        <v>4088</v>
       </c>
       <c r="E389" t="n">
-        <v>2026</v>
+        <v>17086</v>
       </c>
       <c r="F389" t="n">
-        <v>4088</v>
+        <v>16.5</v>
       </c>
       <c r="G389" t="n">
-        <v>17086</v>
+        <v>20.7</v>
       </c>
       <c r="H389" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: fix 180203 zhāoshāng re-parsed rows (label 化 fix, all 20 months corrected)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -6092,16 +6092,16 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>-12.9</v>
+        <v>3470</v>
       </c>
       <c r="E146" t="n">
-        <v>4</v>
+        <v>13462</v>
       </c>
       <c r="F146" t="n">
-        <v>-7.3</v>
+        <v>-4.9</v>
       </c>
       <c r="G146" t="n">
-        <v>-8.5</v>
+        <v>-2.9</v>
       </c>
       <c r="H146" t="inlineStr">
         <is>
@@ -6466,16 +6466,16 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>-4.6</v>
+        <v>3777</v>
       </c>
       <c r="E157" t="n">
-        <v>12</v>
+        <v>13335</v>
       </c>
       <c r="F157" t="n">
-        <v>3.7</v>
+        <v>13.6</v>
       </c>
       <c r="G157" t="n">
-        <v>-3.1</v>
+        <v>10.3</v>
       </c>
       <c r="H157" t="inlineStr">
         <is>
@@ -6874,16 +6874,16 @@
         </is>
       </c>
       <c r="D169" t="n">
+        <v>4357</v>
+      </c>
+      <c r="E169" t="n">
+        <v>20086</v>
+      </c>
+      <c r="F169" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G169" t="n">
         <v>36.6</v>
-      </c>
-      <c r="E169" t="n">
-        <v>1</v>
-      </c>
-      <c r="F169" t="n">
-        <v>15.4</v>
-      </c>
-      <c r="G169" t="n">
-        <v>50.6</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
@@ -7282,16 +7282,16 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>25.4</v>
+        <v>3009</v>
       </c>
       <c r="E181" t="n">
-        <v>2</v>
+        <v>16277</v>
       </c>
       <c r="F181" t="n">
-        <v>-30.9</v>
+        <v>18</v>
       </c>
       <c r="G181" t="n">
-        <v>-19</v>
+        <v>12.9</v>
       </c>
       <c r="H181" t="inlineStr">
         <is>
@@ -7724,16 +7724,16 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>16.2</v>
+        <v>3776</v>
       </c>
       <c r="E194" t="n">
-        <v>3</v>
+        <v>14517</v>
       </c>
       <c r="F194" t="n">
-        <v>25.5</v>
+        <v>0.9</v>
       </c>
       <c r="G194" t="n">
-        <v>-10.8</v>
+        <v>-1.4</v>
       </c>
       <c r="H194" t="inlineStr">
         <is>
@@ -8166,16 +8166,16 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>12.8</v>
+        <v>3589</v>
       </c>
       <c r="E207" t="n">
-        <v>4</v>
+        <v>13697</v>
       </c>
       <c r="F207" t="n">
-        <v>-5</v>
+        <v>3.4</v>
       </c>
       <c r="G207" t="n">
-        <v>-5.6</v>
+        <v>1.7</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
@@ -8608,16 +8608,16 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>11.5</v>
+        <v>3569</v>
       </c>
       <c r="E220" t="n">
-        <v>5</v>
+        <v>13116</v>
       </c>
       <c r="F220" t="n">
-        <v>-0.6</v>
+        <v>5.6</v>
       </c>
       <c r="G220" t="n">
-        <v>-5</v>
+        <v>5.1</v>
       </c>
       <c r="H220" t="inlineStr">
         <is>
@@ -9050,16 +9050,16 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>10.1</v>
+        <v>3508</v>
       </c>
       <c r="E233" t="n">
-        <v>6</v>
+        <v>14153</v>
       </c>
       <c r="F233" t="n">
-        <v>-1.7</v>
+        <v>3.6</v>
       </c>
       <c r="G233" t="n">
-        <v>7.9</v>
+        <v>3.3</v>
       </c>
       <c r="H233" t="inlineStr">
         <is>
@@ -9492,16 +9492,16 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>9.699999999999999</v>
+        <v>3867</v>
       </c>
       <c r="E246" t="n">
-        <v>7</v>
+        <v>15634</v>
       </c>
       <c r="F246" t="n">
-        <v>10.2</v>
+        <v>7.9</v>
       </c>
       <c r="G246" t="n">
-        <v>10.5</v>
+        <v>7.3</v>
       </c>
       <c r="H246" t="inlineStr">
         <is>
@@ -9934,16 +9934,16 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>9.4</v>
+        <v>4087</v>
       </c>
       <c r="E259" t="n">
-        <v>8</v>
+        <v>17173</v>
       </c>
       <c r="F259" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
       <c r="G259" t="n">
-        <v>9.800000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
@@ -10376,16 +10376,16 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>8.699999999999999</v>
+        <v>3962</v>
       </c>
       <c r="E272" t="n">
-        <v>9</v>
+        <v>15930</v>
       </c>
       <c r="F272" t="n">
-        <v>-3</v>
+        <v>4.3</v>
       </c>
       <c r="G272" t="n">
-        <v>-7.2</v>
+        <v>3.5</v>
       </c>
       <c r="H272" t="inlineStr">
         <is>
@@ -10818,16 +10818,16 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>8.4</v>
+        <v>3680</v>
       </c>
       <c r="E285" t="n">
-        <v>10</v>
+        <v>13033</v>
       </c>
       <c r="F285" t="n">
-        <v>-7.1</v>
+        <v>5.1</v>
       </c>
       <c r="G285" t="n">
-        <v>-18.2</v>
+        <v>5.4</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
@@ -11226,16 +11226,16 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>8.6</v>
+        <v>4081</v>
       </c>
       <c r="E297" t="n">
-        <v>11</v>
+        <v>15237</v>
       </c>
       <c r="F297" t="n">
-        <v>10.9</v>
+        <v>12</v>
       </c>
       <c r="G297" t="n">
-        <v>16.9</v>
+        <v>10.7</v>
       </c>
       <c r="H297" t="inlineStr">
         <is>
@@ -11634,16 +11634,16 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>8.699999999999999</v>
+        <v>3952</v>
       </c>
       <c r="E309" t="n">
-        <v>12</v>
+        <v>14645</v>
       </c>
       <c r="F309" t="n">
-        <v>-3.2</v>
+        <v>4.6</v>
       </c>
       <c r="G309" t="n">
-        <v>-3.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H309" t="inlineStr">
         <is>
@@ -12076,16 +12076,16 @@
         </is>
       </c>
       <c r="D322" t="n">
+        <v>4170</v>
+      </c>
+      <c r="E322" t="n">
+        <v>15880</v>
+      </c>
+      <c r="F322" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="G322" t="n">
         <v>-20.9</v>
-      </c>
-      <c r="E322" t="n">
-        <v>1</v>
-      </c>
-      <c r="F322" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="G322" t="n">
-        <v>8.4</v>
       </c>
       <c r="H322" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: fill concession years left (14 funds, verified from public disclosures)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -571,7 +571,9 @@
       <c r="G2" s="2" t="n">
         <v>91.14</v>
       </c>
-      <c r="H2" s="2" t="n"/>
+      <c r="H2" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -610,7 +612,9 @@
       <c r="G3" s="2" t="n">
         <v>21.3</v>
       </c>
-      <c r="H3" s="2" t="n"/>
+      <c r="H3" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -649,7 +653,9 @@
       <c r="G4" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H4" s="2" t="n"/>
+      <c r="H4" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -688,7 +694,9 @@
       <c r="G5" s="2" t="n">
         <v>93.98999999999999</v>
       </c>
-      <c r="H5" s="2" t="n"/>
+      <c r="H5" s="2" t="n">
+        <v>20</v>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -727,7 +735,9 @@
       <c r="G6" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H6" s="2" t="n"/>
+      <c r="H6" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -766,7 +776,9 @@
       <c r="G7" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H7" s="2" t="n"/>
+      <c r="H7" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -805,7 +817,9 @@
       <c r="G8" s="2" t="n">
         <v>108.8</v>
       </c>
-      <c r="H8" s="2" t="n"/>
+      <c r="H8" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -844,7 +858,9 @@
       <c r="G9" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H9" s="2" t="n"/>
+      <c r="H9" s="2" t="n">
+        <v>14</v>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -883,7 +899,9 @@
       <c r="G10" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H10" s="2" t="n"/>
+      <c r="H10" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -922,7 +940,9 @@
       <c r="G11" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="H11" s="2" t="n"/>
+      <c r="H11" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -961,7 +981,9 @@
       <c r="G12" s="2" t="n">
         <v>27.27</v>
       </c>
-      <c r="H12" s="2" t="n"/>
+      <c r="H12" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -1000,7 +1022,9 @@
       <c r="G13" s="2" t="n">
         <v>34.96</v>
       </c>
-      <c r="H13" s="2" t="n"/>
+      <c r="H13" s="2" t="n">
+        <v>10</v>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>高速公路</t>
@@ -1039,7 +1063,9 @@
       <c r="G14" s="2" t="n">
         <v>80.88</v>
       </c>
-      <c r="H14" s="2" t="n"/>
+      <c r="H14" s="2" t="n">
+        <v>7</v>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>桥梁</t>
@@ -1078,7 +1104,9 @@
       <c r="G15" s="2" t="n">
         <v>46.8</v>
       </c>
-      <c r="H15" s="2" t="n"/>
+      <c r="H15" s="2" t="n">
+        <v>13</v>
+      </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
           <t>隧道</t>

</xml_diff>

<commit_message>
data: fix static asset names (180203 亳阜高速, 508020 钱江隧道 per announcements)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -1003,16 +1003,16 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>渝黔高速</t>
+          <t>亳阜高速(安徽)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>西南</t>
+          <t>华东</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>110</v>
+        <v>101.3</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1085,16 +1085,16 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>大连湾海底隧道</t>
+          <t>钱江隧道(钱江通道及接线工程)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>东北</t>
+          <t>华东</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>5</v>
+        <v>4.45</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1113,6 +1113,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: quarterly cost parsing + NAV-based yield KPI
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -1113,7 +1113,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -14868,6 +14867,9 @@
       <c r="D3" t="n">
         <v>17803.43</v>
       </c>
+      <c r="E3" t="n">
+        <v>21270.781361</v>
+      </c>
       <c r="F3" t="n">
         <v>4249.11</v>
       </c>
@@ -14930,6 +14932,9 @@
       <c r="D5" t="n">
         <v>15588.66</v>
       </c>
+      <c r="E5" t="n">
+        <v>25708.089434</v>
+      </c>
       <c r="F5" t="n">
         <v>-5899.29</v>
       </c>
@@ -14992,6 +14997,9 @@
       <c r="D7" t="n">
         <v>5668.96</v>
       </c>
+      <c r="E7" t="n">
+        <v>3066.780922</v>
+      </c>
       <c r="F7" t="n">
         <v>1629.82</v>
       </c>
@@ -15085,6 +15093,9 @@
       <c r="D10" t="n">
         <v>4994.78</v>
       </c>
+      <c r="E10" t="n">
+        <v>2655.903315</v>
+      </c>
       <c r="F10" t="n">
         <v>1184.45</v>
       </c>
@@ -15147,6 +15158,9 @@
       <c r="D12" t="n">
         <v>10628.9</v>
       </c>
+      <c r="E12" t="n">
+        <v>4701.069372</v>
+      </c>
       <c r="F12" t="n">
         <v>3316.44</v>
       </c>
@@ -15209,6 +15223,9 @@
       <c r="D14" t="n">
         <v>5634.12</v>
       </c>
+      <c r="E14" t="n">
+        <v>2206.508136</v>
+      </c>
       <c r="F14" t="n">
         <v>2298.14</v>
       </c>
@@ -15302,6 +15319,9 @@
       <c r="D17" t="n">
         <v>11493.67</v>
       </c>
+      <c r="E17" t="n">
+        <v>5188.082883</v>
+      </c>
       <c r="F17" t="n">
         <v>2730.06</v>
       </c>
@@ -15364,6 +15384,9 @@
       <c r="D19" t="n">
         <v>4563.33</v>
       </c>
+      <c r="E19" t="n">
+        <v>5403.347954</v>
+      </c>
       <c r="F19" t="n">
         <v>-1975.63</v>
       </c>
@@ -15457,6 +15480,9 @@
       <c r="D22" t="n">
         <v>9885.5</v>
       </c>
+      <c r="E22" t="n">
+        <v>5217.226361</v>
+      </c>
       <c r="F22" t="n">
         <v>1911.79</v>
       </c>
@@ -15519,6 +15545,9 @@
       <c r="D24" t="n">
         <v>6531.6</v>
       </c>
+      <c r="E24" t="n">
+        <v>3403.598714</v>
+      </c>
       <c r="F24" t="n">
         <v>1673.09</v>
       </c>
@@ -15612,6 +15641,9 @@
       <c r="D27" t="n">
         <v>26950.74</v>
       </c>
+      <c r="E27" t="n">
+        <v>21221.558927</v>
+      </c>
       <c r="F27" t="n">
         <v>1859.08</v>
       </c>
@@ -15643,6 +15675,9 @@
       <c r="D28" t="n">
         <v>11732.36</v>
       </c>
+      <c r="E28" t="n">
+        <v>5030.611209000001</v>
+      </c>
       <c r="F28" t="n">
         <v>3385.11</v>
       </c>
@@ -15736,6 +15771,9 @@
       <c r="D31" t="n">
         <v>5813.25</v>
       </c>
+      <c r="E31" t="n">
+        <v>3403.953977</v>
+      </c>
       <c r="F31" t="n">
         <v>1208.4</v>
       </c>
@@ -15829,6 +15867,9 @@
       <c r="D34" t="n">
         <v>24304.45</v>
       </c>
+      <c r="E34" t="n">
+        <v>21240.651139</v>
+      </c>
       <c r="F34" t="n">
         <v>-84.68000000000001</v>
       </c>
@@ -15860,6 +15901,9 @@
       <c r="D35" t="n">
         <v>10851.83</v>
       </c>
+      <c r="E35" t="n">
+        <v>5405.807924000001</v>
+      </c>
       <c r="F35" t="n">
         <v>2346.33</v>
       </c>
@@ -15953,6 +15997,9 @@
       <c r="D38" t="n">
         <v>6490.64</v>
       </c>
+      <c r="E38" t="n">
+        <v>3664.441822</v>
+      </c>
       <c r="F38" t="n">
         <v>1412.42</v>
       </c>
@@ -16046,6 +16093,9 @@
       <c r="D41" t="n">
         <v>25826.14</v>
       </c>
+      <c r="E41" t="n">
+        <v>21524.333724</v>
+      </c>
       <c r="F41" t="n">
         <v>846.64</v>
       </c>
@@ -16077,6 +16127,9 @@
       <c r="D42" t="n">
         <v>11813</v>
       </c>
+      <c r="E42" t="n">
+        <v>5535.792544</v>
+      </c>
       <c r="F42" t="n">
         <v>2864.65</v>
       </c>
@@ -16170,6 +16223,9 @@
       <c r="D45" t="n">
         <v>5692.85</v>
       </c>
+      <c r="E45" t="n">
+        <v>3736.779914</v>
+      </c>
       <c r="F45" t="n">
         <v>694.23</v>
       </c>
@@ -16232,6 +16288,9 @@
       <c r="D47" t="n">
         <v>7071.28</v>
       </c>
+      <c r="E47" t="n">
+        <v>3277.84956</v>
+      </c>
       <c r="F47" t="n">
         <v>2754.16</v>
       </c>
@@ -16294,6 +16353,9 @@
       <c r="D49" t="n">
         <v>19944.45</v>
       </c>
+      <c r="E49" t="n">
+        <v>28186.910345</v>
+      </c>
       <c r="F49" t="n">
         <v>-9031.940000000001</v>
       </c>
@@ -16325,6 +16387,9 @@
       <c r="D50" t="n">
         <v>11768.34</v>
       </c>
+      <c r="E50" t="n">
+        <v>5996.717857</v>
+      </c>
       <c r="F50" t="n">
         <v>2488.51</v>
       </c>
@@ -16418,6 +16483,9 @@
       <c r="D53" t="n">
         <v>5828.28</v>
       </c>
+      <c r="E53" t="n">
+        <v>3482.396029</v>
+      </c>
       <c r="F53" t="n">
         <v>1129.56</v>
       </c>
@@ -16480,6 +16548,9 @@
       <c r="D55" t="n">
         <v>7126.68</v>
       </c>
+      <c r="E55" t="n">
+        <v>4710.931939</v>
+      </c>
       <c r="F55" t="n">
         <v>1187.6</v>
       </c>
@@ -16542,6 +16613,9 @@
       <c r="D57" t="n">
         <v>21594.06</v>
       </c>
+      <c r="E57" t="n">
+        <v>21434.115659</v>
+      </c>
       <c r="F57" t="n">
         <v>-2548.1</v>
       </c>
@@ -16573,6 +16647,9 @@
       <c r="D58" t="n">
         <v>10576.76</v>
       </c>
+      <c r="E58" t="n">
+        <v>5790.641922</v>
+      </c>
       <c r="F58" t="n">
         <v>1662.28</v>
       </c>
@@ -16666,6 +16743,9 @@
       <c r="D61" t="n">
         <v>5661.38</v>
       </c>
+      <c r="E61" t="n">
+        <v>3284.064274</v>
+      </c>
       <c r="F61" t="n">
         <v>1186.29</v>
       </c>
@@ -16728,6 +16808,9 @@
       <c r="D63" t="n">
         <v>7454.03</v>
       </c>
+      <c r="E63" t="n">
+        <v>5033.48062</v>
+      </c>
       <c r="F63" t="n">
         <v>1236.82</v>
       </c>
@@ -16790,6 +16873,9 @@
       <c r="D65" t="n">
         <v>19371.26</v>
       </c>
+      <c r="E65" t="n">
+        <v>21565.04297</v>
+      </c>
       <c r="F65" t="n">
         <v>-4344.69</v>
       </c>
@@ -16821,6 +16907,9 @@
       <c r="D66" t="n">
         <v>9682.809999999999</v>
       </c>
+      <c r="E66" t="n">
+        <v>5582.974254</v>
+      </c>
       <c r="F66" t="n">
         <v>1098.55</v>
       </c>
@@ -16852,6 +16941,9 @@
       <c r="D67" t="n">
         <v>8881.35</v>
       </c>
+      <c r="E67" t="n">
+        <v>4292.625435</v>
+      </c>
       <c r="F67" t="n">
         <v>1051.29</v>
       </c>
@@ -16945,6 +17037,9 @@
       <c r="D70" t="n">
         <v>6015.97</v>
       </c>
+      <c r="E70" t="n">
+        <v>3695.790584</v>
+      </c>
       <c r="F70" t="n">
         <v>1100.02</v>
       </c>
@@ -17007,6 +17102,9 @@
       <c r="D72" t="n">
         <v>8220.57</v>
       </c>
+      <c r="E72" t="n">
+        <v>4419.867017</v>
+      </c>
       <c r="F72" t="n">
         <v>3095.45</v>
       </c>
@@ -17069,6 +17167,9 @@
       <c r="D74" t="n">
         <v>21578.76</v>
       </c>
+      <c r="E74" t="n">
+        <v>21706.540231</v>
+      </c>
       <c r="F74" t="n">
         <v>-2141.68</v>
       </c>
@@ -17100,6 +17201,9 @@
       <c r="D75" t="n">
         <v>11549.21</v>
       </c>
+      <c r="E75" t="n">
+        <v>6194.671622999999</v>
+      </c>
       <c r="F75" t="n">
         <v>2082.22</v>
       </c>
@@ -17131,6 +17235,9 @@
       <c r="D76" t="n">
         <v>11191.53</v>
       </c>
+      <c r="E76" t="n">
+        <v>4210.136436</v>
+      </c>
       <c r="F76" t="n">
         <v>7350.23</v>
       </c>
@@ -17193,6 +17300,9 @@
       <c r="D78" t="n">
         <v>15502.82</v>
       </c>
+      <c r="E78" t="n">
+        <v>12226.309919</v>
+      </c>
       <c r="F78" t="n">
         <v>2483.92</v>
       </c>
@@ -17348,6 +17458,9 @@
       <c r="D83" t="n">
         <v>7929.65</v>
       </c>
+      <c r="E83" t="n">
+        <v>4261.9048</v>
+      </c>
       <c r="F83" t="n">
         <v>2079.16</v>
       </c>
@@ -17410,6 +17523,9 @@
       <c r="D85" t="n">
         <v>20127.41</v>
       </c>
+      <c r="E85" t="n">
+        <v>27998.783828</v>
+      </c>
       <c r="F85" t="n">
         <v>-9841.09</v>
       </c>
@@ -17441,6 +17557,9 @@
       <c r="D86" t="n">
         <v>11104.35</v>
       </c>
+      <c r="E86" t="n">
+        <v>612.8219309999999</v>
+      </c>
       <c r="F86" t="n">
         <v>1195.83</v>
       </c>
@@ -17534,6 +17653,9 @@
       <c r="D89" t="n">
         <v>9817.719999999999</v>
       </c>
+      <c r="E89" t="n">
+        <v>490.31617</v>
+      </c>
       <c r="F89" t="n">
         <v>2213.41</v>
       </c>
@@ -17565,6 +17687,9 @@
       <c r="D90" t="n">
         <v>13855.21</v>
       </c>
+      <c r="E90" t="n">
+        <v>12424.027111</v>
+      </c>
       <c r="F90" t="n">
         <v>1957.55</v>
       </c>
@@ -17658,6 +17783,9 @@
       <c r="D93" t="n">
         <v>10909.1</v>
       </c>
+      <c r="E93" t="n">
+        <v>149.093893</v>
+      </c>
       <c r="F93" t="n">
         <v>2370.52</v>
       </c>
@@ -17782,6 +17910,9 @@
       <c r="D97" t="n">
         <v>22975.03</v>
       </c>
+      <c r="E97" t="n">
+        <v>163.49223</v>
+      </c>
       <c r="F97" t="n">
         <v>1241.69</v>
       </c>
@@ -17813,6 +17944,9 @@
       <c r="D98" t="n">
         <v>10849.94</v>
       </c>
+      <c r="E98" t="n">
+        <v>598.141246</v>
+      </c>
       <c r="F98" t="n">
         <v>1512.13</v>
       </c>
@@ -17937,6 +18071,9 @@
       <c r="D102" t="n">
         <v>11255.8</v>
       </c>
+      <c r="E102" t="n">
+        <v>179.81949</v>
+      </c>
       <c r="F102" t="n">
         <v>2910.75</v>
       </c>
@@ -17999,6 +18136,9 @@
       <c r="D104" t="n">
         <v>17174.31</v>
       </c>
+      <c r="E104" t="n">
+        <v>22329.361497</v>
+      </c>
       <c r="F104" t="n">
         <v>4753.3</v>
       </c>
@@ -18067,6 +18207,9 @@
       <c r="D106" t="n">
         <v>10462.18</v>
       </c>
+      <c r="E106" t="n">
+        <v>5351.015711</v>
+      </c>
       <c r="F106" t="n">
         <v>2149.39</v>
       </c>
@@ -18101,6 +18244,9 @@
       <c r="D107" t="n">
         <v>15481.21</v>
       </c>
+      <c r="E107" t="n">
+        <v>19851.538131</v>
+      </c>
       <c r="F107" t="n">
         <v>-266.92</v>
       </c>
@@ -18135,6 +18281,9 @@
       <c r="D108" t="n">
         <v>6538.66</v>
       </c>
+      <c r="E108" t="n">
+        <v>11511.496189</v>
+      </c>
       <c r="F108" t="n">
         <v>1721.68</v>
       </c>
@@ -18169,6 +18318,9 @@
       <c r="D109" t="n">
         <v>17346.05</v>
       </c>
+      <c r="E109" t="n">
+        <v>17475.854087</v>
+      </c>
       <c r="F109" t="n">
         <v>2562.95</v>
       </c>
@@ -18203,6 +18355,9 @@
       <c r="D110" t="n">
         <v>22559.34</v>
       </c>
+      <c r="E110" t="n">
+        <v>39970.099999</v>
+      </c>
       <c r="F110" t="n">
         <v>-304.91</v>
       </c>
@@ -18237,6 +18392,9 @@
       <c r="D111" t="n">
         <v>9656.040000000001</v>
       </c>
+      <c r="E111" t="n">
+        <v>17545.330954</v>
+      </c>
       <c r="F111" t="n">
         <v>928.64</v>
       </c>
@@ -18271,6 +18429,9 @@
       <c r="D112" t="n">
         <v>7856.07</v>
       </c>
+      <c r="E112" t="n">
+        <v>9365.143154000001</v>
+      </c>
       <c r="F112" t="n">
         <v>2408.44</v>
       </c>
@@ -18305,6 +18466,9 @@
       <c r="D113" t="n">
         <v>53501.22</v>
       </c>
+      <c r="E113" t="n">
+        <v>21994.876157</v>
+      </c>
       <c r="F113" t="n">
         <v>11324.73</v>
       </c>
@@ -18339,6 +18503,9 @@
       <c r="D114" t="n">
         <v>10240</v>
       </c>
+      <c r="E114" t="n">
+        <v>13335.642566</v>
+      </c>
       <c r="F114" t="n">
         <v>1886.82</v>
       </c>
@@ -18373,6 +18540,9 @@
       <c r="D115" t="n">
         <v>12330.24</v>
       </c>
+      <c r="E115" t="n">
+        <v>24118.36449</v>
+      </c>
       <c r="F115" t="n">
         <v>1951.15</v>
       </c>
@@ -18407,6 +18577,9 @@
       <c r="D116" t="n">
         <v>12774.44</v>
       </c>
+      <c r="E116" t="n">
+        <v>22179.561274</v>
+      </c>
       <c r="F116" t="n">
         <v>225.84</v>
       </c>
@@ -18441,6 +18614,9 @@
       <c r="D117" t="n">
         <v>20153.19</v>
       </c>
+      <c r="E117" t="n">
+        <v>23486.345559</v>
+      </c>
       <c r="F117" t="n">
         <v>6580.56</v>
       </c>
@@ -18475,6 +18651,9 @@
       <c r="D118" t="n">
         <v>5894.58</v>
       </c>
+      <c r="E118" t="n">
+        <v>8133.099074</v>
+      </c>
       <c r="F118" t="n">
         <v>978.4400000000001</v>
       </c>
@@ -18509,6 +18688,9 @@
       <c r="D119" t="n">
         <v>11653.69</v>
       </c>
+      <c r="E119" t="n">
+        <v>5885.467932</v>
+      </c>
       <c r="F119" t="n">
         <v>2911.71</v>
       </c>
@@ -18543,6 +18725,9 @@
       <c r="D120" t="n">
         <v>19345.62</v>
       </c>
+      <c r="E120" t="n">
+        <v>23734.62151</v>
+      </c>
       <c r="F120" t="n">
         <v>-155.74</v>
       </c>
@@ -18577,6 +18762,9 @@
       <c r="D121" t="n">
         <v>6660.28</v>
       </c>
+      <c r="E121" t="n">
+        <v>9487.585073999999</v>
+      </c>
       <c r="F121" t="n">
         <v>2089.62</v>
       </c>
@@ -18611,6 +18799,9 @@
       <c r="D122" t="n">
         <v>16489.3</v>
       </c>
+      <c r="E122" t="n">
+        <v>17780.997451</v>
+      </c>
       <c r="F122" t="n">
         <v>1527.75</v>
       </c>
@@ -18645,6 +18836,9 @@
       <c r="D123" t="n">
         <v>23283.35</v>
       </c>
+      <c r="E123" t="n">
+        <v>40321.468433</v>
+      </c>
       <c r="F123" t="n">
         <v>306.59</v>
       </c>
@@ -18679,6 +18873,9 @@
       <c r="D124" t="n">
         <v>10769.46</v>
       </c>
+      <c r="E124" t="n">
+        <v>18065.20075</v>
+      </c>
       <c r="F124" t="n">
         <v>2580.41</v>
       </c>
@@ -18713,6 +18910,9 @@
       <c r="D125" t="n">
         <v>9391.129999999999</v>
       </c>
+      <c r="E125" t="n">
+        <v>10263.247926</v>
+      </c>
       <c r="F125" t="n">
         <v>3242.53</v>
       </c>
@@ -18747,6 +18947,9 @@
       <c r="D126" t="n">
         <v>59128.56</v>
       </c>
+      <c r="E126" t="n">
+        <v>25986.715704</v>
+      </c>
       <c r="F126" t="n">
         <v>13423.06</v>
       </c>
@@ -18781,6 +18984,9 @@
       <c r="D127" t="n">
         <v>12392.76</v>
       </c>
+      <c r="E127" t="n">
+        <v>16416.243909</v>
+      </c>
       <c r="F127" t="n">
         <v>989.8200000000001</v>
       </c>
@@ -18815,6 +19021,9 @@
       <c r="D128" t="n">
         <v>13275.91</v>
       </c>
+      <c r="E128" t="n">
+        <v>19654.561205</v>
+      </c>
       <c r="F128" t="n">
         <v>3751.71</v>
       </c>
@@ -18849,6 +19058,9 @@
       <c r="D129" t="n">
         <v>15907.47</v>
       </c>
+      <c r="E129" t="n">
+        <v>16450.279081</v>
+      </c>
       <c r="F129" t="n">
         <v>3112.01</v>
       </c>
@@ -18883,6 +19095,9 @@
       <c r="D130" t="n">
         <v>17706.85</v>
       </c>
+      <c r="E130" t="n">
+        <v>23262.429491</v>
+      </c>
       <c r="F130" t="n">
         <v>4145.78</v>
       </c>
@@ -18917,6 +19132,9 @@
       <c r="D131" t="n">
         <v>5281.55</v>
       </c>
+      <c r="E131" t="n">
+        <v>8389.358998</v>
+      </c>
       <c r="F131" t="n">
         <v>340.4</v>
       </c>
@@ -18951,6 +19169,9 @@
       <c r="D132" t="n">
         <v>11547.58</v>
       </c>
+      <c r="E132" t="n">
+        <v>5641.158898</v>
+      </c>
       <c r="F132" t="n">
         <v>3175.65</v>
       </c>
@@ -18985,6 +19206,9 @@
       <c r="D133" t="n">
         <v>16407.93</v>
       </c>
+      <c r="E133" t="n">
+        <v>23318.630017</v>
+      </c>
       <c r="F133" t="n">
         <v>-2672.76</v>
       </c>
@@ -19019,6 +19243,9 @@
       <c r="D134" t="n">
         <v>6334.83</v>
       </c>
+      <c r="E134" t="n">
+        <v>7241.850231999999</v>
+      </c>
       <c r="F134" t="n">
         <v>752.25</v>
       </c>
@@ -19053,6 +19280,9 @@
       <c r="D135" t="n">
         <v>16106.02</v>
       </c>
+      <c r="E135" t="n">
+        <v>18975.413234</v>
+      </c>
       <c r="F135" t="n">
         <v>287.1</v>
       </c>
@@ -19087,6 +19317,9 @@
       <c r="D136" t="n">
         <v>19673.66</v>
       </c>
+      <c r="E136" t="n">
+        <v>44175.59864</v>
+      </c>
       <c r="F136" t="n">
         <v>-7156.57</v>
       </c>
@@ -19121,6 +19354,9 @@
       <c r="D137" t="n">
         <v>10908.52</v>
       </c>
+      <c r="E137" t="n">
+        <v>18872.859956</v>
+      </c>
       <c r="F137" t="n">
         <v>1909.16</v>
       </c>
@@ -19155,6 +19391,9 @@
       <c r="D138" t="n">
         <v>8415.02</v>
       </c>
+      <c r="E138" t="n">
+        <v>18053.480641</v>
+      </c>
       <c r="F138" t="n">
         <v>-1475.61</v>
       </c>
@@ -19189,6 +19428,9 @@
       <c r="D139" t="n">
         <v>54769.26</v>
       </c>
+      <c r="E139" t="n">
+        <v>36148.49027</v>
+      </c>
       <c r="F139" t="n">
         <v>3529.42</v>
       </c>
@@ -19223,6 +19465,9 @@
       <c r="D140" t="n">
         <v>12617.78</v>
       </c>
+      <c r="E140" t="n">
+        <v>14895.476576</v>
+      </c>
       <c r="F140" t="n">
         <v>2700.74</v>
       </c>
@@ -19257,6 +19502,9 @@
       <c r="D141" t="n">
         <v>12149.46</v>
       </c>
+      <c r="E141" t="n">
+        <v>21302.363649</v>
+      </c>
       <c r="F141" t="n">
         <v>837.05</v>
       </c>
@@ -19291,6 +19539,9 @@
       <c r="D142" t="n">
         <v>12685.92</v>
       </c>
+      <c r="E142" t="n">
+        <v>16267.731464</v>
+      </c>
       <c r="F142" t="n">
         <v>-219.11</v>
       </c>
@@ -19325,6 +19576,9 @@
       <c r="D143" t="n">
         <v>18563.69</v>
       </c>
+      <c r="E143" t="n">
+        <v>22590.245374</v>
+      </c>
       <c r="F143" t="n">
         <v>5434.94</v>
       </c>
@@ -19359,6 +19613,9 @@
       <c r="D144" t="n">
         <v>6119.44</v>
       </c>
+      <c r="E144" t="n">
+        <v>8253.415123000001</v>
+      </c>
       <c r="F144" t="n">
         <v>995.5599999999999</v>
       </c>
@@ -19393,6 +19650,9 @@
       <c r="D145" t="n">
         <v>12655.9</v>
       </c>
+      <c r="E145" t="n">
+        <v>5801.578452000001</v>
+      </c>
       <c r="F145" t="n">
         <v>3637.84</v>
       </c>
@@ -19427,6 +19687,9 @@
       <c r="D146" t="n">
         <v>18574.52</v>
       </c>
+      <c r="E146" t="n">
+        <v>20591.817239</v>
+      </c>
       <c r="F146" t="n">
         <v>1924.56</v>
       </c>
@@ -19461,6 +19724,9 @@
       <c r="D147" t="n">
         <v>5762.94</v>
       </c>
+      <c r="E147" t="n">
+        <v>7262.955928</v>
+      </c>
       <c r="F147" t="n">
         <v>1497.65</v>
       </c>
@@ -19495,6 +19761,9 @@
       <c r="D148" t="n">
         <v>16342.13</v>
       </c>
+      <c r="E148" t="n">
+        <v>16988.262617</v>
+      </c>
       <c r="F148" t="n">
         <v>1928.1</v>
       </c>
@@ -19529,6 +19798,9 @@
       <c r="D149" t="n">
         <v>20052.7</v>
       </c>
+      <c r="E149" t="n">
+        <v>35930.947415</v>
+      </c>
       <c r="F149" t="n">
         <v>-1482.25</v>
       </c>
@@ -19563,6 +19835,9 @@
       <c r="D150" t="n">
         <v>11942.83</v>
       </c>
+      <c r="E150" t="n">
+        <v>18180.872673</v>
+      </c>
       <c r="F150" t="n">
         <v>2826.67</v>
       </c>
@@ -19597,6 +19872,9 @@
       <c r="D151" t="n">
         <v>9543.860000000001</v>
       </c>
+      <c r="E151" t="n">
+        <v>4562.89282</v>
+      </c>
       <c r="F151" t="n">
         <v>1901.53</v>
       </c>
@@ -19631,6 +19909,9 @@
       <c r="D152" t="n">
         <v>48091.49</v>
       </c>
+      <c r="E152" t="n">
+        <v>22586.03843</v>
+      </c>
       <c r="F152" t="n">
         <v>9354.459999999999</v>
       </c>
@@ -19665,6 +19946,9 @@
       <c r="D153" t="n">
         <v>12282.91</v>
       </c>
+      <c r="E153" t="n">
+        <v>12976.259903</v>
+      </c>
       <c r="F153" t="n">
         <v>4269.24</v>
       </c>
@@ -19699,6 +19983,9 @@
       <c r="D154" t="n">
         <v>11483.61</v>
       </c>
+      <c r="E154" t="n">
+        <v>15849.904786</v>
+      </c>
       <c r="F154" t="n">
         <v>2566.64</v>
       </c>
@@ -19733,6 +20020,9 @@
       <c r="D155" t="n">
         <v>10335</v>
       </c>
+      <c r="E155" t="n">
+        <v>15969.2342</v>
+      </c>
       <c r="F155" t="n">
         <v>-2205.09</v>
       </c>
@@ -19767,6 +20057,9 @@
       <c r="D156" t="n">
         <v>16539.13</v>
       </c>
+      <c r="E156" t="n">
+        <v>23043.990264</v>
+      </c>
       <c r="F156" t="n">
         <v>3032.1</v>
       </c>
@@ -19801,6 +20094,9 @@
       <c r="D157" t="n">
         <v>5324.92</v>
       </c>
+      <c r="E157" t="n">
+        <v>8225.665182999999</v>
+      </c>
       <c r="F157" t="n">
         <v>414.48</v>
       </c>
@@ -19835,6 +20131,9 @@
       <c r="D158" t="n">
         <v>11891.96</v>
       </c>
+      <c r="E158" t="n">
+        <v>5299.125546</v>
+      </c>
       <c r="F158" t="n">
         <v>3652.59</v>
       </c>
@@ -19869,6 +20168,9 @@
       <c r="D159" t="n">
         <v>16029.59</v>
       </c>
+      <c r="E159" t="n">
+        <v>4073.621506</v>
+      </c>
       <c r="F159" t="n">
         <v>-476.76</v>
       </c>
@@ -19903,6 +20205,9 @@
       <c r="D160" t="n">
         <v>6099.53</v>
       </c>
+      <c r="E160" t="n">
+        <v>7212.603195999999</v>
+      </c>
       <c r="F160" t="n">
         <v>1544.54</v>
       </c>
@@ -19937,6 +20242,9 @@
       <c r="D161" t="n">
         <v>15562.19</v>
       </c>
+      <c r="E161" t="n">
+        <v>17545.652648</v>
+      </c>
       <c r="F161" t="n">
         <v>943.42</v>
       </c>
@@ -19971,6 +20279,9 @@
       <c r="D162" t="n">
         <v>21124.22</v>
       </c>
+      <c r="E162" t="n">
+        <v>36537.296493</v>
+      </c>
       <c r="F162" t="n">
         <v>-838.05</v>
       </c>
@@ -20005,6 +20316,9 @@
       <c r="D163" t="n">
         <v>11195.48</v>
       </c>
+      <c r="E163" t="n">
+        <v>17929.637411</v>
+      </c>
       <c r="F163" t="n">
         <v>2480.29</v>
       </c>
@@ -20039,6 +20353,9 @@
       <c r="D164" t="n">
         <v>13583.85</v>
       </c>
+      <c r="E164" t="n">
+        <v>5701.272639</v>
+      </c>
       <c r="F164" t="n">
         <v>3434.73</v>
       </c>
@@ -20073,6 +20390,9 @@
       <c r="D165" t="n">
         <v>7745.39</v>
       </c>
+      <c r="E165" t="n">
+        <v>3940.119391</v>
+      </c>
       <c r="F165" t="n">
         <v>1176.47</v>
       </c>
@@ -20107,6 +20427,9 @@
       <c r="D166" t="n">
         <v>53483.86</v>
       </c>
+      <c r="E166" t="n">
+        <v>27343.664814</v>
+      </c>
       <c r="F166" t="n">
         <v>9227.09</v>
       </c>
@@ -20141,6 +20464,9 @@
       <c r="D167" t="n">
         <v>13611.88</v>
       </c>
+      <c r="E167" t="n">
+        <v>14959.055165</v>
+      </c>
       <c r="F167" t="n">
         <v>3598.25</v>
       </c>
@@ -20175,6 +20501,9 @@
       <c r="D168" t="n">
         <v>11309.01</v>
       </c>
+      <c r="E168" t="n">
+        <v>16570.399295</v>
+      </c>
       <c r="F168" t="n">
         <v>1769.8</v>
       </c>
@@ -20208,6 +20537,9 @@
       </c>
       <c r="D169" t="n">
         <v>10901.2</v>
+      </c>
+      <c r="E169" t="n">
+        <v>15667.389863</v>
       </c>
       <c r="F169" t="n">
         <v>-1277.49</v>

</xml_diff>

<commit_message>
data: backfill NAV from annual reports (ffill by year)
</commit_message>
<xml_diff>
--- a/data/REITsMonitor_数据模板_v1.xlsx
+++ b/data/REITsMonitor_数据模板_v1.xlsx
@@ -14907,6 +14907,9 @@
       <c r="G4" t="n">
         <v>17161.79</v>
       </c>
+      <c r="I4" t="n">
+        <v>887511.63</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -14941,6 +14944,9 @@
       <c r="G5" t="n">
         <v>4409.26</v>
       </c>
+      <c r="I5" t="n">
+        <v>417491.28</v>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -14972,6 +14978,9 @@
       <c r="G6" t="n">
         <v>10593.44</v>
       </c>
+      <c r="I6" t="n">
+        <v>887511.63</v>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15037,6 +15046,9 @@
       <c r="G8" t="n">
         <v>11523.44</v>
       </c>
+      <c r="I8" t="n">
+        <v>417491.28</v>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15068,6 +15080,9 @@
       <c r="G9" t="n">
         <v>12663.51</v>
       </c>
+      <c r="I9" t="n">
+        <v>887511.63</v>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15133,6 +15148,9 @@
       <c r="G11" t="n">
         <v>7502.39</v>
       </c>
+      <c r="I11" t="n">
+        <v>417491.28</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15198,6 +15216,9 @@
       <c r="G13" t="n">
         <v>17671.41</v>
       </c>
+      <c r="I13" t="n">
+        <v>887511.63</v>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15263,6 +15284,9 @@
       <c r="G15" t="n">
         <v>10460.17</v>
       </c>
+      <c r="I15" t="n">
+        <v>417491.28</v>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15359,6 +15383,9 @@
       <c r="G18" t="n">
         <v>9214.5</v>
       </c>
+      <c r="I18" t="n">
+        <v>860066.41</v>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15393,6 +15420,9 @@
       <c r="G19" t="n">
         <v>2905.31</v>
       </c>
+      <c r="I19" t="n">
+        <v>208223.78</v>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15424,6 +15454,9 @@
       <c r="G20" t="n">
         <v>2383.02</v>
       </c>
+      <c r="I20" t="n">
+        <v>371633.97</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15455,6 +15488,9 @@
       <c r="G21" t="n">
         <v>7907.73</v>
       </c>
+      <c r="I21" t="n">
+        <v>478747.48</v>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15489,6 +15525,9 @@
       <c r="G22" t="n">
         <v>7276.81</v>
       </c>
+      <c r="I22" t="n">
+        <v>927505.37</v>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15520,6 +15559,9 @@
       <c r="G23" t="n">
         <v>14803.06</v>
       </c>
+      <c r="I23" t="n">
+        <v>860066.41</v>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15554,6 +15596,9 @@
       <c r="G24" t="n">
         <v>4433.37</v>
       </c>
+      <c r="I24" t="n">
+        <v>208223.78</v>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15585,6 +15630,9 @@
       <c r="G25" t="n">
         <v>13946.01</v>
       </c>
+      <c r="I25" t="n">
+        <v>371633.97</v>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15616,6 +15664,9 @@
       <c r="G26" t="n">
         <v>14561.18</v>
       </c>
+      <c r="I26" t="n">
+        <v>478747.48</v>
+      </c>
       <c r="J26" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15684,6 +15735,9 @@
       <c r="G28" t="n">
         <v>9339.85</v>
       </c>
+      <c r="I28" t="n">
+        <v>927505.37</v>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15746,6 +15800,9 @@
       <c r="G30" t="n">
         <v>10664.12</v>
       </c>
+      <c r="I30" t="n">
+        <v>860066.41</v>
+      </c>
       <c r="J30" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15780,6 +15837,9 @@
       <c r="G31" t="n">
         <v>3779.11</v>
       </c>
+      <c r="I31" t="n">
+        <v>208223.78</v>
+      </c>
       <c r="J31" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15811,6 +15871,9 @@
       <c r="G32" t="n">
         <v>10861.88</v>
       </c>
+      <c r="I32" t="n">
+        <v>371633.97</v>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15842,6 +15905,9 @@
       <c r="G33" t="n">
         <v>12530.42</v>
       </c>
+      <c r="I33" t="n">
+        <v>478747.48</v>
+      </c>
       <c r="J33" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15910,6 +15976,9 @@
       <c r="G35" t="n">
         <v>7044.05</v>
       </c>
+      <c r="I35" t="n">
+        <v>927505.37</v>
+      </c>
       <c r="J35" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -15972,6 +16041,9 @@
       <c r="G37" t="n">
         <v>17005.47</v>
       </c>
+      <c r="I37" t="n">
+        <v>860066.41</v>
+      </c>
       <c r="J37" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16006,6 +16078,9 @@
       <c r="G38" t="n">
         <v>4274.56</v>
       </c>
+      <c r="I38" t="n">
+        <v>208223.78</v>
+      </c>
       <c r="J38" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16037,6 +16112,9 @@
       <c r="G39" t="n">
         <v>14831.55</v>
       </c>
+      <c r="I39" t="n">
+        <v>371633.97</v>
+      </c>
       <c r="J39" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16068,6 +16146,9 @@
       <c r="G40" t="n">
         <v>13833.07</v>
       </c>
+      <c r="I40" t="n">
+        <v>478747.48</v>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16136,6 +16217,9 @@
       <c r="G42" t="n">
         <v>7888.27</v>
       </c>
+      <c r="I42" t="n">
+        <v>927505.37</v>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16198,6 +16282,9 @@
       <c r="G44" t="n">
         <v>11899.55</v>
       </c>
+      <c r="I44" t="n">
+        <v>817472.9300000001</v>
+      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16232,6 +16319,9 @@
       <c r="G45" t="n">
         <v>3922.45</v>
       </c>
+      <c r="I45" t="n">
+        <v>194235.66</v>
+      </c>
       <c r="J45" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16263,6 +16353,9 @@
       <c r="G46" t="n">
         <v>5659.51</v>
       </c>
+      <c r="I46" t="n">
+        <v>343894.6</v>
+      </c>
       <c r="J46" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16297,6 +16390,9 @@
       <c r="G47" t="n">
         <v>35621.77</v>
       </c>
+      <c r="I47" t="n">
+        <v>277117.76</v>
+      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16328,6 +16424,9 @@
       <c r="G48" t="n">
         <v>7908.18</v>
       </c>
+      <c r="I48" t="n">
+        <v>453528.66</v>
+      </c>
       <c r="J48" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16362,6 +16461,9 @@
       <c r="G49" t="n">
         <v>18423.32</v>
       </c>
+      <c r="I49" t="n">
+        <v>972712.38</v>
+      </c>
       <c r="J49" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16396,6 +16498,9 @@
       <c r="G50" t="n">
         <v>7763.64</v>
       </c>
+      <c r="I50" t="n">
+        <v>906030.3199999999</v>
+      </c>
       <c r="J50" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16427,6 +16532,9 @@
       <c r="G51" t="n">
         <v>4277.76</v>
       </c>
+      <c r="I51" t="n">
+        <v>202266.19</v>
+      </c>
       <c r="J51" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16458,6 +16566,9 @@
       <c r="G52" t="n">
         <v>15110.76</v>
       </c>
+      <c r="I52" t="n">
+        <v>817472.9300000001</v>
+      </c>
       <c r="J52" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16492,6 +16603,9 @@
       <c r="G53" t="n">
         <v>3398.73</v>
       </c>
+      <c r="I53" t="n">
+        <v>194235.66</v>
+      </c>
       <c r="J53" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16523,6 +16637,9 @@
       <c r="G54" t="n">
         <v>14499.52</v>
       </c>
+      <c r="I54" t="n">
+        <v>343894.6</v>
+      </c>
       <c r="J54" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16557,6 +16674,9 @@
       <c r="G55" t="n">
         <v>4904.75</v>
       </c>
+      <c r="I55" t="n">
+        <v>277117.76</v>
+      </c>
       <c r="J55" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16588,6 +16708,9 @@
       <c r="G56" t="n">
         <v>12406.89</v>
       </c>
+      <c r="I56" t="n">
+        <v>453528.66</v>
+      </c>
       <c r="J56" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16622,6 +16745,9 @@
       <c r="G57" t="n">
         <v>12942.32</v>
       </c>
+      <c r="I57" t="n">
+        <v>972712.38</v>
+      </c>
       <c r="J57" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16656,6 +16782,9 @@
       <c r="G58" t="n">
         <v>7200.34</v>
       </c>
+      <c r="I58" t="n">
+        <v>906030.3199999999</v>
+      </c>
       <c r="J58" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16687,6 +16816,9 @@
       <c r="G59" t="n">
         <v>7026.31</v>
       </c>
+      <c r="I59" t="n">
+        <v>202266.19</v>
+      </c>
       <c r="J59" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16718,6 +16850,9 @@
       <c r="G60" t="n">
         <v>10648.83</v>
       </c>
+      <c r="I60" t="n">
+        <v>817472.9300000001</v>
+      </c>
       <c r="J60" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16752,6 +16887,9 @@
       <c r="G61" t="n">
         <v>3149.88</v>
       </c>
+      <c r="I61" t="n">
+        <v>194235.66</v>
+      </c>
       <c r="J61" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16783,6 +16921,9 @@
       <c r="G62" t="n">
         <v>6893.16</v>
       </c>
+      <c r="I62" t="n">
+        <v>343894.6</v>
+      </c>
       <c r="J62" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16817,6 +16958,9 @@
       <c r="G63" t="n">
         <v>4776.98</v>
       </c>
+      <c r="I63" t="n">
+        <v>277117.76</v>
+      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16848,6 +16992,9 @@
       <c r="G64" t="n">
         <v>11538.58</v>
       </c>
+      <c r="I64" t="n">
+        <v>453528.66</v>
+      </c>
       <c r="J64" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16882,6 +17029,9 @@
       <c r="G65" t="n">
         <v>16310.62</v>
       </c>
+      <c r="I65" t="n">
+        <v>972712.38</v>
+      </c>
       <c r="J65" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16916,6 +17066,9 @@
       <c r="G66" t="n">
         <v>6084.84</v>
       </c>
+      <c r="I66" t="n">
+        <v>906030.3199999999</v>
+      </c>
       <c r="J66" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -16981,6 +17134,9 @@
       <c r="G68" t="n">
         <v>5716.18</v>
       </c>
+      <c r="I68" t="n">
+        <v>202266.19</v>
+      </c>
       <c r="J68" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17012,6 +17168,9 @@
       <c r="G69" t="n">
         <v>17271.71</v>
       </c>
+      <c r="I69" t="n">
+        <v>817472.9300000001</v>
+      </c>
       <c r="J69" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17046,6 +17205,9 @@
       <c r="G70" t="n">
         <v>3786.75</v>
       </c>
+      <c r="I70" t="n">
+        <v>194235.66</v>
+      </c>
       <c r="J70" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17077,6 +17239,9 @@
       <c r="G71" t="n">
         <v>12776.64</v>
       </c>
+      <c r="I71" t="n">
+        <v>343894.6</v>
+      </c>
       <c r="J71" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17111,6 +17276,9 @@
       <c r="G72" t="n">
         <v>4961.21</v>
       </c>
+      <c r="I72" t="n">
+        <v>277117.76</v>
+      </c>
       <c r="J72" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17142,6 +17310,9 @@
       <c r="G73" t="n">
         <v>14454.79</v>
       </c>
+      <c r="I73" t="n">
+        <v>453528.66</v>
+      </c>
       <c r="J73" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17176,6 +17347,9 @@
       <c r="G74" t="n">
         <v>18345.26</v>
       </c>
+      <c r="I74" t="n">
+        <v>972712.38</v>
+      </c>
       <c r="J74" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17210,6 +17384,9 @@
       <c r="G75" t="n">
         <v>7839.85</v>
       </c>
+      <c r="I75" t="n">
+        <v>906030.3199999999</v>
+      </c>
       <c r="J75" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17275,6 +17452,9 @@
       <c r="G77" t="n">
         <v>6211.98</v>
       </c>
+      <c r="I77" t="n">
+        <v>202266.19</v>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17340,6 +17520,9 @@
       <c r="G79" t="n">
         <v>9601.059999999999</v>
       </c>
+      <c r="I79" t="n">
+        <v>734851.28</v>
+      </c>
       <c r="J79" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17371,6 +17554,9 @@
       <c r="G80" t="n">
         <v>2460.41</v>
       </c>
+      <c r="I80" t="n">
+        <v>183155.86</v>
+      </c>
       <c r="J80" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17402,6 +17588,9 @@
       <c r="G81" t="n">
         <v>23534.74</v>
       </c>
+      <c r="I81" t="n">
+        <v>330634.18</v>
+      </c>
       <c r="J81" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17433,6 +17622,9 @@
       <c r="G82" t="n">
         <v>8818.84</v>
       </c>
+      <c r="I82" t="n">
+        <v>280767.53</v>
+      </c>
       <c r="J82" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17467,6 +17659,9 @@
       <c r="G83" t="n">
         <v>4228.8</v>
       </c>
+      <c r="I83" t="n">
+        <v>257418.97</v>
+      </c>
       <c r="J83" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17498,6 +17693,9 @@
       <c r="G84" t="n">
         <v>9319.040000000001</v>
       </c>
+      <c r="I84" t="n">
+        <v>393615.94</v>
+      </c>
       <c r="J84" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17532,6 +17730,9 @@
       <c r="G85" t="n">
         <v>12436.42</v>
       </c>
+      <c r="I85" t="n">
+        <v>793688.34</v>
+      </c>
       <c r="J85" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17566,6 +17767,9 @@
       <c r="G86" t="n">
         <v>5351.87</v>
       </c>
+      <c r="I86" t="n">
+        <v>759969.65</v>
+      </c>
       <c r="J86" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17597,6 +17801,9 @@
       <c r="G87" t="n">
         <v>4785.24</v>
       </c>
+      <c r="I87" t="n">
+        <v>187514.29</v>
+      </c>
       <c r="J87" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17628,6 +17835,9 @@
       <c r="G88" t="n">
         <v>3824.61</v>
       </c>
+      <c r="I88" t="n">
+        <v>179319.88</v>
+      </c>
       <c r="J88" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17662,6 +17872,9 @@
       <c r="G89" t="n">
         <v>17676.11</v>
       </c>
+      <c r="I89" t="n">
+        <v>273988.58</v>
+      </c>
       <c r="J89" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17696,6 +17909,9 @@
       <c r="G90" t="n">
         <v>11651.54</v>
       </c>
+      <c r="I90" t="n">
+        <v>534166.17</v>
+      </c>
       <c r="J90" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17727,6 +17943,9 @@
       <c r="G91" t="n">
         <v>15103.64</v>
       </c>
+      <c r="I91" t="n">
+        <v>734851.28</v>
+      </c>
       <c r="J91" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17758,6 +17977,9 @@
       <c r="G92" t="n">
         <v>2691.95</v>
       </c>
+      <c r="I92" t="n">
+        <v>183155.86</v>
+      </c>
       <c r="J92" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17792,6 +18014,9 @@
       <c r="G93" t="n">
         <v>7951.29</v>
       </c>
+      <c r="I93" t="n">
+        <v>330634.18</v>
+      </c>
       <c r="J93" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17823,6 +18048,9 @@
       <c r="G94" t="n">
         <v>13996.32</v>
       </c>
+      <c r="I94" t="n">
+        <v>280767.53</v>
+      </c>
       <c r="J94" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17854,6 +18082,9 @@
       <c r="G95" t="n">
         <v>4905.98</v>
       </c>
+      <c r="I95" t="n">
+        <v>257418.97</v>
+      </c>
       <c r="J95" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17885,6 +18116,9 @@
       <c r="G96" t="n">
         <v>10561.13</v>
       </c>
+      <c r="I96" t="n">
+        <v>393615.94</v>
+      </c>
       <c r="J96" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17919,6 +18153,9 @@
       <c r="G97" t="n">
         <v>16761.54</v>
       </c>
+      <c r="I97" t="n">
+        <v>793688.34</v>
+      </c>
       <c r="J97" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17953,6 +18190,9 @@
       <c r="G98" t="n">
         <v>7263.88</v>
       </c>
+      <c r="I98" t="n">
+        <v>759969.65</v>
+      </c>
       <c r="J98" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -17984,6 +18224,9 @@
       <c r="G99" t="n">
         <v>5812.93</v>
       </c>
+      <c r="I99" t="n">
+        <v>187514.29</v>
+      </c>
       <c r="J99" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18046,6 +18289,9 @@
       <c r="G101" t="n">
         <v>7609.39</v>
       </c>
+      <c r="I101" t="n">
+        <v>179319.88</v>
+      </c>
       <c r="J101" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18080,6 +18326,9 @@
       <c r="G102" t="n">
         <v>6824.63</v>
       </c>
+      <c r="I102" t="n">
+        <v>273988.58</v>
+      </c>
       <c r="J102" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18111,6 +18360,9 @@
       <c r="G103" t="n">
         <v>8116.84</v>
       </c>
+      <c r="I103" t="n">
+        <v>534166.17</v>
+      </c>
       <c r="J103" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18148,6 +18400,9 @@
       <c r="H104" t="n">
         <v>14146.05</v>
       </c>
+      <c r="I104" t="n">
+        <v>734851.28</v>
+      </c>
       <c r="J104" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18182,6 +18437,9 @@
       <c r="H105" t="n">
         <v>4311.01</v>
       </c>
+      <c r="I105" t="n">
+        <v>183155.86</v>
+      </c>
       <c r="J105" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18219,6 +18477,9 @@
       <c r="H106" t="n">
         <v>8783.92</v>
       </c>
+      <c r="I106" t="n">
+        <v>330634.18</v>
+      </c>
       <c r="J106" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18256,6 +18517,9 @@
       <c r="H107" t="n">
         <v>12743.05</v>
       </c>
+      <c r="I107" t="n">
+        <v>280767.53</v>
+      </c>
       <c r="J107" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18293,6 +18557,9 @@
       <c r="H108" t="n">
         <v>5123.41</v>
       </c>
+      <c r="I108" t="n">
+        <v>257418.97</v>
+      </c>
       <c r="J108" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18330,6 +18597,9 @@
       <c r="H109" t="n">
         <v>14736.19</v>
       </c>
+      <c r="I109" t="n">
+        <v>393615.94</v>
+      </c>
       <c r="J109" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18367,6 +18637,9 @@
       <c r="H110" t="n">
         <v>18963.31</v>
       </c>
+      <c r="I110" t="n">
+        <v>793688.34</v>
+      </c>
       <c r="J110" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18404,6 +18677,9 @@
       <c r="H111" t="n">
         <v>7526.52</v>
       </c>
+      <c r="I111" t="n">
+        <v>759969.65</v>
+      </c>
       <c r="J111" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18441,6 +18717,9 @@
       <c r="H112" t="n">
         <v>6525.04</v>
       </c>
+      <c r="I112" t="n">
+        <v>187514.29</v>
+      </c>
       <c r="J112" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18515,6 +18794,9 @@
       <c r="H114" t="n">
         <v>7823.52</v>
       </c>
+      <c r="I114" t="n">
+        <v>179319.88</v>
+      </c>
       <c r="J114" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18552,6 +18834,9 @@
       <c r="H115" t="n">
         <v>8181.37</v>
       </c>
+      <c r="I115" t="n">
+        <v>273988.58</v>
+      </c>
       <c r="J115" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18589,6 +18874,9 @@
       <c r="H116" t="n">
         <v>11222.95</v>
       </c>
+      <c r="I116" t="n">
+        <v>534166.17</v>
+      </c>
       <c r="J116" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18626,6 +18914,9 @@
       <c r="H117" t="n">
         <v>17330.54</v>
       </c>
+      <c r="I117" t="n">
+        <v>734851.28</v>
+      </c>
       <c r="J117" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18663,6 +18954,9 @@
       <c r="H118" t="n">
         <v>4961.16</v>
       </c>
+      <c r="I118" t="n">
+        <v>183155.86</v>
+      </c>
       <c r="J118" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18700,6 +18994,9 @@
       <c r="H119" t="n">
         <v>9893.84</v>
       </c>
+      <c r="I119" t="n">
+        <v>330634.18</v>
+      </c>
       <c r="J119" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18737,6 +19034,9 @@
       <c r="H120" t="n">
         <v>12977.24</v>
       </c>
+      <c r="I120" t="n">
+        <v>280767.53</v>
+      </c>
       <c r="J120" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18774,6 +19074,9 @@
       <c r="H121" t="n">
         <v>5534.71</v>
       </c>
+      <c r="I121" t="n">
+        <v>257418.97</v>
+      </c>
       <c r="J121" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18811,6 +19114,9 @@
       <c r="H122" t="n">
         <v>13600.7</v>
       </c>
+      <c r="I122" t="n">
+        <v>393615.94</v>
+      </c>
       <c r="J122" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18848,6 +19154,9 @@
       <c r="H123" t="n">
         <v>19557.49</v>
       </c>
+      <c r="I123" t="n">
+        <v>793688.34</v>
+      </c>
       <c r="J123" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18885,6 +19194,9 @@
       <c r="H124" t="n">
         <v>8607.25</v>
       </c>
+      <c r="I124" t="n">
+        <v>759969.65</v>
+      </c>
       <c r="J124" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18922,6 +19234,9 @@
       <c r="H125" t="n">
         <v>8068.13</v>
       </c>
+      <c r="I125" t="n">
+        <v>187514.29</v>
+      </c>
       <c r="J125" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -18996,6 +19311,9 @@
       <c r="H127" t="n">
         <v>6143.53</v>
       </c>
+      <c r="I127" t="n">
+        <v>179319.88</v>
+      </c>
       <c r="J127" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19033,6 +19351,9 @@
       <c r="H128" t="n">
         <v>9544.309999999999</v>
       </c>
+      <c r="I128" t="n">
+        <v>273988.58</v>
+      </c>
       <c r="J128" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19070,6 +19391,9 @@
       <c r="H129" t="n">
         <v>13899.15</v>
       </c>
+      <c r="I129" t="n">
+        <v>534166.17</v>
+      </c>
       <c r="J129" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19107,6 +19431,9 @@
       <c r="H130" t="n">
         <v>14134.48</v>
       </c>
+      <c r="I130" t="n">
+        <v>700438.4300000001</v>
+      </c>
       <c r="J130" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19144,6 +19471,9 @@
       <c r="H131" t="n">
         <v>4255.01</v>
       </c>
+      <c r="I131" t="n">
+        <v>174584.72</v>
+      </c>
       <c r="J131" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19181,6 +19511,9 @@
       <c r="H132" t="n">
         <v>9763.950000000001</v>
       </c>
+      <c r="I132" t="n">
+        <v>309856.31</v>
+      </c>
       <c r="J132" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19218,6 +19551,9 @@
       <c r="H133" t="n">
         <v>10498.21</v>
       </c>
+      <c r="I133" t="n">
+        <v>238154.3</v>
+      </c>
       <c r="J133" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19255,6 +19591,9 @@
       <c r="H134" t="n">
         <v>3588.18</v>
       </c>
+      <c r="I134" t="n">
+        <v>245062.99</v>
+      </c>
       <c r="J134" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19292,6 +19631,9 @@
       <c r="H135" t="n">
         <v>11844.04</v>
       </c>
+      <c r="I135" t="n">
+        <v>354353.11</v>
+      </c>
       <c r="J135" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19329,6 +19671,9 @@
       <c r="H136" t="n">
         <v>12102.35</v>
       </c>
+      <c r="I136" t="n">
+        <v>725866.39</v>
+      </c>
       <c r="J136" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19366,6 +19711,9 @@
       <c r="H137" t="n">
         <v>7964.01</v>
       </c>
+      <c r="I137" t="n">
+        <v>740355.87</v>
+      </c>
       <c r="J137" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19403,6 +19751,9 @@
       <c r="H138" t="n">
         <v>4942.64</v>
       </c>
+      <c r="I138" t="n">
+        <v>169713.76</v>
+      </c>
       <c r="J138" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19440,6 +19791,9 @@
       <c r="H139" t="n">
         <v>38657.96</v>
       </c>
+      <c r="I139" t="n">
+        <v>730759.41</v>
+      </c>
       <c r="J139" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19477,6 +19831,9 @@
       <c r="H140" t="n">
         <v>8749.1</v>
       </c>
+      <c r="I140" t="n">
+        <v>162873.76</v>
+      </c>
       <c r="J140" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19514,6 +19871,9 @@
       <c r="H141" t="n">
         <v>8489.290000000001</v>
       </c>
+      <c r="I141" t="n">
+        <v>244847.87</v>
+      </c>
       <c r="J141" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19551,6 +19911,9 @@
       <c r="H142" t="n">
         <v>10806.59</v>
       </c>
+      <c r="I142" t="n">
+        <v>486418.54</v>
+      </c>
       <c r="J142" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19588,6 +19951,9 @@
       <c r="H143" t="n">
         <v>16532.57</v>
       </c>
+      <c r="I143" t="n">
+        <v>700438.4300000001</v>
+      </c>
       <c r="J143" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19625,6 +19991,9 @@
       <c r="H144" t="n">
         <v>5145.59</v>
       </c>
+      <c r="I144" t="n">
+        <v>174584.72</v>
+      </c>
       <c r="J144" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19662,6 +20031,9 @@
       <c r="H145" t="n">
         <v>11050.72</v>
       </c>
+      <c r="I145" t="n">
+        <v>309856.31</v>
+      </c>
       <c r="J145" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19699,6 +20071,9 @@
       <c r="H146" t="n">
         <v>14968.01</v>
       </c>
+      <c r="I146" t="n">
+        <v>238154.3</v>
+      </c>
       <c r="J146" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19736,6 +20111,9 @@
       <c r="H147" t="n">
         <v>4456.12</v>
       </c>
+      <c r="I147" t="n">
+        <v>245062.99</v>
+      </c>
       <c r="J147" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19773,6 +20151,9 @@
       <c r="H148" t="n">
         <v>14078.43</v>
       </c>
+      <c r="I148" t="n">
+        <v>354353.11</v>
+      </c>
       <c r="J148" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19810,6 +20191,9 @@
       <c r="H149" t="n">
         <v>17651.09</v>
       </c>
+      <c r="I149" t="n">
+        <v>725866.39</v>
+      </c>
       <c r="J149" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19847,6 +20231,9 @@
       <c r="H150" t="n">
         <v>10025.19</v>
       </c>
+      <c r="I150" t="n">
+        <v>740355.87</v>
+      </c>
       <c r="J150" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19884,6 +20271,9 @@
       <c r="H151" t="n">
         <v>8366.1</v>
       </c>
+      <c r="I151" t="n">
+        <v>169713.76</v>
+      </c>
       <c r="J151" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19921,6 +20311,9 @@
       <c r="H152" t="n">
         <v>44108.14</v>
       </c>
+      <c r="I152" t="n">
+        <v>730759.41</v>
+      </c>
       <c r="J152" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19958,6 +20351,9 @@
       <c r="H153" t="n">
         <v>10213.09</v>
       </c>
+      <c r="I153" t="n">
+        <v>162873.76</v>
+      </c>
       <c r="J153" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -19995,6 +20391,9 @@
       <c r="H154" t="n">
         <v>8369.620000000001</v>
       </c>
+      <c r="I154" t="n">
+        <v>244847.87</v>
+      </c>
       <c r="J154" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20032,6 +20431,9 @@
       <c r="H155" t="n">
         <v>8570.59</v>
       </c>
+      <c r="I155" t="n">
+        <v>486418.54</v>
+      </c>
       <c r="J155" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20069,6 +20471,9 @@
       <c r="H156" t="n">
         <v>13618.28</v>
       </c>
+      <c r="I156" t="n">
+        <v>700438.4300000001</v>
+      </c>
       <c r="J156" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20106,6 +20511,9 @@
       <c r="H157" t="n">
         <v>4392.49</v>
       </c>
+      <c r="I157" t="n">
+        <v>174584.72</v>
+      </c>
       <c r="J157" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20143,6 +20551,9 @@
       <c r="H158" t="n">
         <v>10300.21</v>
       </c>
+      <c r="I158" t="n">
+        <v>309856.31</v>
+      </c>
       <c r="J158" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20180,6 +20591,9 @@
       <c r="H159" t="n">
         <v>13007.83</v>
       </c>
+      <c r="I159" t="n">
+        <v>238154.3</v>
+      </c>
       <c r="J159" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20217,6 +20631,9 @@
       <c r="H160" t="n">
         <v>4979.86</v>
       </c>
+      <c r="I160" t="n">
+        <v>245062.99</v>
+      </c>
       <c r="J160" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20254,6 +20671,9 @@
       <c r="H161" t="n">
         <v>12812.05</v>
       </c>
+      <c r="I161" t="n">
+        <v>354353.11</v>
+      </c>
       <c r="J161" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20291,6 +20711,9 @@
       <c r="H162" t="n">
         <v>18306.9</v>
       </c>
+      <c r="I162" t="n">
+        <v>725866.39</v>
+      </c>
       <c r="J162" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20328,6 +20751,9 @@
       <c r="H163" t="n">
         <v>9384.639999999999</v>
       </c>
+      <c r="I163" t="n">
+        <v>740355.87</v>
+      </c>
       <c r="J163" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20402,6 +20828,9 @@
       <c r="H165" t="n">
         <v>6570.19</v>
       </c>
+      <c r="I165" t="n">
+        <v>169713.76</v>
+      </c>
       <c r="J165" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20439,6 +20868,9 @@
       <c r="H166" t="n">
         <v>46204.68</v>
       </c>
+      <c r="I166" t="n">
+        <v>730759.41</v>
+      </c>
       <c r="J166" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20476,6 +20908,9 @@
       <c r="H167" t="n">
         <v>9628.059999999999</v>
       </c>
+      <c r="I167" t="n">
+        <v>162873.76</v>
+      </c>
       <c r="J167" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20513,6 +20948,9 @@
       <c r="H168" t="n">
         <v>7779.96</v>
       </c>
+      <c r="I168" t="n">
+        <v>244847.87</v>
+      </c>
       <c r="J168" t="inlineStr">
         <is>
           <t>季度报告（自动采集）</t>
@@ -20549,6 +20987,9 @@
       </c>
       <c r="H169" t="n">
         <v>9457.92</v>
+      </c>
+      <c r="I169" t="n">
+        <v>486418.54</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>

</xml_diff>